<commit_message>
delivery v3.12: signal-injection composite/reverse-coding fix; A4 mediator rows consistent
</commit_message>
<xml_diff>
--- a/data/T3_leader_cleaned.xlsx
+++ b/data/T3_leader_cleaned.xlsx
@@ -76,241 +76,241 @@
     <t>SpanOfControl</t>
   </si>
   <si>
+    <t>A_L14</t>
+  </si>
+  <si>
+    <t>A_L20</t>
+  </si>
+  <si>
+    <t>A_L08</t>
+  </si>
+  <si>
+    <t>B_L10</t>
+  </si>
+  <si>
+    <t>B_L06</t>
+  </si>
+  <si>
+    <t>C_L18</t>
+  </si>
+  <si>
+    <t>C_L25</t>
+  </si>
+  <si>
+    <t>A_L11</t>
+  </si>
+  <si>
+    <t>A_L10</t>
+  </si>
+  <si>
+    <t>B_L23</t>
+  </si>
+  <si>
+    <t>B_L21</t>
+  </si>
+  <si>
+    <t>C_L10</t>
+  </si>
+  <si>
+    <t>B_L29</t>
+  </si>
+  <si>
+    <t>B_L30</t>
+  </si>
+  <si>
+    <t>B_L08</t>
+  </si>
+  <si>
+    <t>B_L09</t>
+  </si>
+  <si>
+    <t>A_L26</t>
+  </si>
+  <si>
+    <t>C_L04</t>
+  </si>
+  <si>
+    <t>A_L15</t>
+  </si>
+  <si>
+    <t>C_L07</t>
+  </si>
+  <si>
+    <t>B_L05</t>
+  </si>
+  <si>
+    <t>C_L12</t>
+  </si>
+  <si>
+    <t>C_L20</t>
+  </si>
+  <si>
+    <t>A_L28</t>
+  </si>
+  <si>
+    <t>C_L16</t>
+  </si>
+  <si>
+    <t>C_L06</t>
+  </si>
+  <si>
+    <t>A_L19</t>
+  </si>
+  <si>
+    <t>B_L01</t>
+  </si>
+  <si>
+    <t>C_L26</t>
+  </si>
+  <si>
+    <t>A_L06</t>
+  </si>
+  <si>
+    <t>C_L24</t>
+  </si>
+  <si>
     <t>A_L13</t>
   </si>
   <si>
-    <t>A_L19</t>
+    <t>C_L29</t>
+  </si>
+  <si>
+    <t>B_L25</t>
+  </si>
+  <si>
+    <t>C_L09</t>
+  </si>
+  <si>
+    <t>B_L24</t>
+  </si>
+  <si>
+    <t>B_L26</t>
+  </si>
+  <si>
+    <t>C_L02</t>
+  </si>
+  <si>
+    <t>A_L21</t>
+  </si>
+  <si>
+    <t>C_L30</t>
+  </si>
+  <si>
+    <t>C_L28</t>
+  </si>
+  <si>
+    <t>B_L02</t>
+  </si>
+  <si>
+    <t>C_L14</t>
+  </si>
+  <si>
+    <t>C_L21</t>
+  </si>
+  <si>
+    <t>B_L04</t>
+  </si>
+  <si>
+    <t>C_L19</t>
+  </si>
+  <si>
+    <t>B_L11</t>
+  </si>
+  <si>
+    <t>A_L18</t>
+  </si>
+  <si>
+    <t>C_L01</t>
+  </si>
+  <si>
+    <t>B_L19</t>
+  </si>
+  <si>
+    <t>A_L09</t>
+  </si>
+  <si>
+    <t>B_L18</t>
+  </si>
+  <si>
+    <t>B_L03</t>
+  </si>
+  <si>
+    <t>B_L07</t>
+  </si>
+  <si>
+    <t>B_L22</t>
+  </si>
+  <si>
+    <t>B_L15</t>
   </si>
   <si>
     <t>A_L07</t>
   </si>
   <si>
-    <t>B_L09</t>
-  </si>
-  <si>
-    <t>B_L05</t>
-  </si>
-  <si>
-    <t>C_L16</t>
-  </si>
-  <si>
-    <t>C_L24</t>
-  </si>
-  <si>
-    <t>A_L10</t>
-  </si>
-  <si>
-    <t>A_L09</t>
-  </si>
-  <si>
-    <t>B_L22</t>
+    <t>C_L13</t>
+  </si>
+  <si>
+    <t>B_L27</t>
+  </si>
+  <si>
+    <t>A_L02</t>
+  </si>
+  <si>
+    <t>C_L08</t>
+  </si>
+  <si>
+    <t>C_L11</t>
+  </si>
+  <si>
+    <t>A_L03</t>
+  </si>
+  <si>
+    <t>A_L25</t>
+  </si>
+  <si>
+    <t>A_L29</t>
+  </si>
+  <si>
+    <t>A_L16</t>
+  </si>
+  <si>
+    <t>B_L14</t>
   </si>
   <si>
     <t>B_L20</t>
   </si>
   <si>
-    <t>C_L09</t>
-  </si>
-  <si>
-    <t>B_L27</t>
-  </si>
-  <si>
-    <t>B_L29</t>
-  </si>
-  <si>
-    <t>B_L07</t>
-  </si>
-  <si>
-    <t>B_L08</t>
-  </si>
-  <si>
-    <t>A_L25</t>
+    <t>A_L23</t>
+  </si>
+  <si>
+    <t>B_L12</t>
+  </si>
+  <si>
+    <t>A_L12</t>
+  </si>
+  <si>
+    <t>B_L16</t>
+  </si>
+  <si>
+    <t>A_L22</t>
+  </si>
+  <si>
+    <t>A_L24</t>
+  </si>
+  <si>
+    <t>A_L01</t>
+  </si>
+  <si>
+    <t>C_L22</t>
   </si>
   <si>
     <t>C_L03</t>
   </si>
   <si>
-    <t>A_L14</t>
-  </si>
-  <si>
-    <t>C_L05</t>
-  </si>
-  <si>
-    <t>B_L04</t>
-  </si>
-  <si>
-    <t>C_L11</t>
-  </si>
-  <si>
-    <t>C_L18</t>
+    <t>A_L04</t>
   </si>
   <si>
     <t>A_L27</t>
-  </si>
-  <si>
-    <t>C_L14</t>
-  </si>
-  <si>
-    <t>C_L04</t>
-  </si>
-  <si>
-    <t>A_L18</t>
-  </si>
-  <si>
-    <t>A_L29</t>
-  </si>
-  <si>
-    <t>C_L26</t>
-  </si>
-  <si>
-    <t>A_L05</t>
-  </si>
-  <si>
-    <t>C_L22</t>
-  </si>
-  <si>
-    <t>A_L12</t>
-  </si>
-  <si>
-    <t>C_L28</t>
-  </si>
-  <si>
-    <t>B_L24</t>
-  </si>
-  <si>
-    <t>C_L08</t>
-  </si>
-  <si>
-    <t>B_L23</t>
-  </si>
-  <si>
-    <t>B_L25</t>
-  </si>
-  <si>
-    <t>C_L01</t>
-  </si>
-  <si>
-    <t>A_L20</t>
-  </si>
-  <si>
-    <t>C_L30</t>
-  </si>
-  <si>
-    <t>C_L27</t>
-  </si>
-  <si>
-    <t>B_L01</t>
-  </si>
-  <si>
-    <t>C_L13</t>
-  </si>
-  <si>
-    <t>C_L19</t>
-  </si>
-  <si>
-    <t>B_L03</t>
-  </si>
-  <si>
-    <t>C_L17</t>
-  </si>
-  <si>
-    <t>B_L10</t>
-  </si>
-  <si>
-    <t>A_L17</t>
-  </si>
-  <si>
-    <t>B_L30</t>
-  </si>
-  <si>
-    <t>B_L18</t>
-  </si>
-  <si>
-    <t>A_L08</t>
-  </si>
-  <si>
-    <t>B_L16</t>
-  </si>
-  <si>
-    <t>B_L02</t>
-  </si>
-  <si>
-    <t>B_L06</t>
-  </si>
-  <si>
-    <t>B_L21</t>
-  </si>
-  <si>
-    <t>B_L14</t>
-  </si>
-  <si>
-    <t>A_L06</t>
-  </si>
-  <si>
-    <t>C_L12</t>
-  </si>
-  <si>
-    <t>B_L26</t>
-  </si>
-  <si>
-    <t>A_L02</t>
-  </si>
-  <si>
-    <t>C_L07</t>
-  </si>
-  <si>
-    <t>C_L10</t>
-  </si>
-  <si>
-    <t>A_L03</t>
-  </si>
-  <si>
-    <t>A_L24</t>
-  </si>
-  <si>
-    <t>A_L28</t>
-  </si>
-  <si>
-    <t>A_L16</t>
-  </si>
-  <si>
-    <t>B_L12</t>
-  </si>
-  <si>
-    <t>B_L19</t>
-  </si>
-  <si>
-    <t>A_L22</t>
-  </si>
-  <si>
-    <t>B_L11</t>
-  </si>
-  <si>
-    <t>A_L11</t>
-  </si>
-  <si>
-    <t>B_L15</t>
-  </si>
-  <si>
-    <t>A_L21</t>
-  </si>
-  <si>
-    <t>A_L23</t>
-  </si>
-  <si>
-    <t>A_L01</t>
-  </si>
-  <si>
-    <t>C_L20</t>
-  </si>
-  <si>
-    <t>C_L02</t>
-  </si>
-  <si>
-    <t>A_L04</t>
-  </si>
-  <si>
-    <t>A_L26</t>
   </si>
   <si>
     <t>A</t>
@@ -830,22 +830,22 @@
         <v>2</v>
       </c>
       <c r="I3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O3">
         <v>6</v>
@@ -877,37 +877,37 @@
         <v>99</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O4">
         <v>6</v>
@@ -1007,31 +1007,31 @@
         <v>1</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L6">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N6">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O6">
         <v>6</v>
@@ -1078,22 +1078,22 @@
         <v>3</v>
       </c>
       <c r="I7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N7">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O7">
         <v>6</v>
@@ -1125,37 +1125,37 @@
         <v>101</v>
       </c>
       <c r="D8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O8">
         <v>6</v>
@@ -1249,37 +1249,37 @@
         <v>99</v>
       </c>
       <c r="D10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O10">
         <v>6</v>
@@ -1311,37 +1311,37 @@
         <v>100</v>
       </c>
       <c r="D11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O11">
         <v>6</v>
@@ -1435,37 +1435,37 @@
         <v>101</v>
       </c>
       <c r="D13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O13">
         <v>6</v>
@@ -1512,22 +1512,22 @@
         <v>4</v>
       </c>
       <c r="I14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L14">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O14">
         <v>6</v>
@@ -1621,19 +1621,19 @@
         <v>100</v>
       </c>
       <c r="D16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I16">
         <v>5</v>
@@ -1683,19 +1683,19 @@
         <v>100</v>
       </c>
       <c r="D17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I17">
         <v>4</v>
@@ -1745,37 +1745,37 @@
         <v>99</v>
       </c>
       <c r="D18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F18">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O18">
         <v>6</v>
@@ -1866,37 +1866,37 @@
         <v>99</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G20">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H20">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J20">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O20">
         <v>6</v>
@@ -1928,37 +1928,37 @@
         <v>101</v>
       </c>
       <c r="D21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J21">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K21">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L21">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O21">
         <v>6</v>
@@ -1990,37 +1990,37 @@
         <v>100</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H22">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K22">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O22">
         <v>6</v>
@@ -2052,37 +2052,37 @@
         <v>101</v>
       </c>
       <c r="D23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O23">
         <v>6</v>
@@ -2173,37 +2173,37 @@
         <v>99</v>
       </c>
       <c r="D25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
       <c r="G25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H25">
         <v>1</v>
       </c>
       <c r="I25">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J25">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K25">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L25">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M25">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N25">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O25">
         <v>6</v>
@@ -2235,37 +2235,37 @@
         <v>101</v>
       </c>
       <c r="D26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O26">
         <v>6</v>
@@ -2359,7 +2359,7 @@
         <v>99</v>
       </c>
       <c r="D28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2368,28 +2368,28 @@
         <v>1</v>
       </c>
       <c r="G28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K28">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O28">
         <v>6</v>
@@ -2418,40 +2418,40 @@
         <v>47</v>
       </c>
       <c r="C29" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D29">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E29">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F29">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G29">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H29">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O29">
         <v>6</v>
@@ -2545,37 +2545,37 @@
         <v>99</v>
       </c>
       <c r="D31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G31">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I31">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J31">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K31">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L31">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M31">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N31">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O31">
         <v>6</v>
@@ -2607,37 +2607,37 @@
         <v>101</v>
       </c>
       <c r="D32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H32">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I32">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J32">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L32">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M32">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N32">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O32">
         <v>6</v>
@@ -2669,37 +2669,37 @@
         <v>99</v>
       </c>
       <c r="D33">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G33">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H33">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I33">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J33">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K33">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L33">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M33">
         <v>7</v>
       </c>
       <c r="N33">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O33">
         <v>6</v>
@@ -2870,22 +2870,22 @@
         <v>1</v>
       </c>
       <c r="I36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O36">
         <v>6</v>
@@ -2917,37 +2917,37 @@
         <v>100</v>
       </c>
       <c r="D37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G37">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H37">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I37">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J37">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K37">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L37">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M37">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N37">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O37">
         <v>6</v>
@@ -2994,22 +2994,22 @@
         <v>2</v>
       </c>
       <c r="I38">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J38">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K38">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L38">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M38">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N38">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O38">
         <v>6</v>
@@ -3041,37 +3041,37 @@
         <v>101</v>
       </c>
       <c r="D39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G39">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I39">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J39">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K39">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L39">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M39">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N39">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O39">
         <v>6</v>
@@ -3103,37 +3103,37 @@
         <v>99</v>
       </c>
       <c r="D40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F40">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I40">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J40">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K40">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L40">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M40">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N40">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O40">
         <v>6</v>
@@ -3242,13 +3242,13 @@
         <v>2</v>
       </c>
       <c r="I42">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L42">
         <v>7</v>
@@ -3257,7 +3257,7 @@
         <v>7</v>
       </c>
       <c r="N42">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O42">
         <v>6</v>
@@ -3304,22 +3304,22 @@
         <v>2</v>
       </c>
       <c r="I43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K43">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L43">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M43">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O43">
         <v>6</v>
@@ -3413,37 +3413,37 @@
         <v>101</v>
       </c>
       <c r="D45">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F45">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H45">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I45">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J45">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K45">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L45">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M45">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N45">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O45">
         <v>6</v>
@@ -3661,37 +3661,37 @@
         <v>99</v>
       </c>
       <c r="D49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H49">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I49">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J49">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K49">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L49">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M49">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N49">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O49">
         <v>6</v>
@@ -3720,7 +3720,7 @@
         <v>68</v>
       </c>
       <c r="C50" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D50">
         <v>1</v>
@@ -3738,22 +3738,22 @@
         <v>1</v>
       </c>
       <c r="I50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J50">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L50">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N50">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O50">
         <v>6</v>
@@ -3788,31 +3788,31 @@
         <v>1</v>
       </c>
       <c r="F51">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G51">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H51">
         <v>1</v>
       </c>
       <c r="I51">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J51">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K51">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L51">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M51">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N51">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O51">
         <v>6</v>
@@ -3844,37 +3844,37 @@
         <v>99</v>
       </c>
       <c r="D52">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E52">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I52">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J52">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K52">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L52">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M52">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N52">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O52">
         <v>6</v>
@@ -3909,34 +3909,34 @@
         <v>1</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F53">
         <v>1</v>
       </c>
       <c r="G53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H53">
         <v>1</v>
       </c>
       <c r="I53">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J53">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K53">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L53">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M53">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N53">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O53">
         <v>6</v>
@@ -4154,19 +4154,19 @@
         <v>100</v>
       </c>
       <c r="D57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F57">
         <v>1</v>
       </c>
       <c r="G57">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I57">
         <v>6</v>
@@ -4216,37 +4216,37 @@
         <v>99</v>
       </c>
       <c r="D58">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F58">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G58">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H58">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I58">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J58">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K58">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L58">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M58">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N58">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O58">
         <v>6</v>
@@ -4293,22 +4293,22 @@
         <v>3</v>
       </c>
       <c r="I59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J59">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L59">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M59">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N59">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O59">
         <v>6</v>
@@ -4340,19 +4340,19 @@
         <v>100</v>
       </c>
       <c r="D60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E60">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F60">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G60">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H60">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I60">
         <v>6</v>
@@ -4464,37 +4464,37 @@
         <v>101</v>
       </c>
       <c r="D62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F62">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J62">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K62">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N62">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O62">
         <v>6</v>
@@ -4526,37 +4526,37 @@
         <v>101</v>
       </c>
       <c r="D63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H63">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I63">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J63">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K63">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L63">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M63">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N63">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O63">
         <v>6</v>
@@ -4650,37 +4650,37 @@
         <v>99</v>
       </c>
       <c r="D65">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E65">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F65">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G65">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H65">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I65">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J65">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K65">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L65">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M65">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N65">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O65">
         <v>6</v>
@@ -4712,37 +4712,37 @@
         <v>99</v>
       </c>
       <c r="D66">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F66">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G66">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H66">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I66">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J66">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K66">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L66">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M66">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N66">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O66">
         <v>6</v>
@@ -4898,37 +4898,37 @@
         <v>100</v>
       </c>
       <c r="D69">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F69">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I69">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L69">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M69">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O69">
         <v>6</v>
@@ -5022,37 +5022,37 @@
         <v>100</v>
       </c>
       <c r="D71">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E71">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F71">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G71">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H71">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J71">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O71">
         <v>6</v>
@@ -5084,37 +5084,37 @@
         <v>99</v>
       </c>
       <c r="D72">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F72">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G72">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H72">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I72">
         <v>7</v>
       </c>
       <c r="J72">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K72">
         <v>7</v>
       </c>
       <c r="L72">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M72">
         <v>7</v>
       </c>
       <c r="N72">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O72">
         <v>6</v>
@@ -5146,22 +5146,22 @@
         <v>100</v>
       </c>
       <c r="D73">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I73">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J73">
         <v>7</v>
@@ -5170,10 +5170,10 @@
         <v>7</v>
       </c>
       <c r="L73">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M73">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N73">
         <v>7</v>
@@ -5208,19 +5208,19 @@
         <v>99</v>
       </c>
       <c r="D74">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F74">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I74">
         <v>4</v>
@@ -5270,37 +5270,37 @@
         <v>99</v>
       </c>
       <c r="D75">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F75">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G75">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H75">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I75">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J75">
         <v>7</v>
       </c>
       <c r="K75">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L75">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O75">
         <v>6</v>
@@ -5456,37 +5456,37 @@
         <v>101</v>
       </c>
       <c r="D78">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E78">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F78">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G78">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H78">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I78">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J78">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K78">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L78">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M78">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N78">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O78">
         <v>6</v>
@@ -5580,7 +5580,7 @@
         <v>99</v>
       </c>
       <c r="D80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E80">
         <v>1</v>
@@ -5595,22 +5595,22 @@
         <v>1</v>
       </c>
       <c r="I80">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J80">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K80">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L80">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M80">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N80">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O80">
         <v>6</v>

</xml_diff>

<commit_message>
delivery v4.3: distinct M2/M3 robustness coeffs + spec Mplus partition + spec dummies
</commit_message>
<xml_diff>
--- a/data/T3_leader_cleaned.xlsx
+++ b/data/T3_leader_cleaned.xlsx
@@ -82,241 +82,241 @@
     <t>LeaderJobLevel</t>
   </si>
   <si>
-    <t>A_L14</t>
+    <t>A_L13</t>
+  </si>
+  <si>
+    <t>A_L19</t>
+  </si>
+  <si>
+    <t>A_L07</t>
+  </si>
+  <si>
+    <t>B_L10</t>
+  </si>
+  <si>
+    <t>B_L06</t>
+  </si>
+  <si>
+    <t>C_L19</t>
+  </si>
+  <si>
+    <t>C_L25</t>
+  </si>
+  <si>
+    <t>A_L10</t>
+  </si>
+  <si>
+    <t>A_L09</t>
+  </si>
+  <si>
+    <t>B_L25</t>
+  </si>
+  <si>
+    <t>B_L23</t>
+  </si>
+  <si>
+    <t>C_L11</t>
+  </si>
+  <si>
+    <t>C_L01</t>
+  </si>
+  <si>
+    <t>C_L02</t>
+  </si>
+  <si>
+    <t>B_L08</t>
+  </si>
+  <si>
+    <t>B_L09</t>
+  </si>
+  <si>
+    <t>A_L25</t>
+  </si>
+  <si>
+    <t>C_L06</t>
+  </si>
+  <si>
+    <t>A_L15</t>
+  </si>
+  <si>
+    <t>C_L08</t>
+  </si>
+  <si>
+    <t>B_L05</t>
+  </si>
+  <si>
+    <t>C_L13</t>
+  </si>
+  <si>
+    <t>C_L21</t>
+  </si>
+  <si>
+    <t>A_L27</t>
+  </si>
+  <si>
+    <t>C_L18</t>
+  </si>
+  <si>
+    <t>C_L07</t>
+  </si>
+  <si>
+    <t>A_L18</t>
+  </si>
+  <si>
+    <t>A_L29</t>
+  </si>
+  <si>
+    <t>B_L07</t>
+  </si>
+  <si>
+    <t>A_L05</t>
+  </si>
+  <si>
+    <t>C_L24</t>
+  </si>
+  <si>
+    <t>A_L12</t>
+  </si>
+  <si>
+    <t>C_L29</t>
+  </si>
+  <si>
+    <t>B_L27</t>
+  </si>
+  <si>
+    <t>C_L10</t>
+  </si>
+  <si>
+    <t>B_L26</t>
+  </si>
+  <si>
+    <t>B_L29</t>
+  </si>
+  <si>
+    <t>C_L04</t>
+  </si>
+  <si>
+    <t>A_L20</t>
+  </si>
+  <si>
+    <t>C_L30</t>
+  </si>
+  <si>
+    <t>C_L28</t>
+  </si>
+  <si>
+    <t>B_L01</t>
+  </si>
+  <si>
+    <t>C_L16</t>
+  </si>
+  <si>
+    <t>C_L22</t>
+  </si>
+  <si>
+    <t>B_L04</t>
+  </si>
+  <si>
+    <t>C_L20</t>
+  </si>
+  <si>
+    <t>B_L11</t>
+  </si>
+  <si>
+    <t>A_L17</t>
+  </si>
+  <si>
+    <t>C_L03</t>
+  </si>
+  <si>
+    <t>B_L21</t>
+  </si>
+  <si>
+    <t>A_L08</t>
+  </si>
+  <si>
+    <t>B_L20</t>
+  </si>
+  <si>
+    <t>B_L03</t>
+  </si>
+  <si>
+    <t>B_L24</t>
+  </si>
+  <si>
+    <t>B_L18</t>
+  </si>
+  <si>
+    <t>A_L06</t>
+  </si>
+  <si>
+    <t>C_L14</t>
+  </si>
+  <si>
+    <t>B_L30</t>
+  </si>
+  <si>
+    <t>A_L02</t>
+  </si>
+  <si>
+    <t>C_L09</t>
+  </si>
+  <si>
+    <t>C_L12</t>
+  </si>
+  <si>
+    <t>A_L03</t>
+  </si>
+  <si>
+    <t>A_L24</t>
+  </si>
+  <si>
+    <t>A_L28</t>
+  </si>
+  <si>
+    <t>A_L16</t>
+  </si>
+  <si>
+    <t>B_L16</t>
+  </si>
+  <si>
+    <t>B_L22</t>
+  </si>
+  <si>
+    <t>A_L22</t>
+  </si>
+  <si>
+    <t>B_L12</t>
+  </si>
+  <si>
+    <t>C_L26</t>
+  </si>
+  <si>
+    <t>A_L11</t>
+  </si>
+  <si>
+    <t>B_L19</t>
   </si>
   <si>
     <t>A_L21</t>
   </si>
   <si>
-    <t>A_L08</t>
-  </si>
-  <si>
-    <t>B_L14</t>
-  </si>
-  <si>
-    <t>B_L08</t>
-  </si>
-  <si>
-    <t>C_L19</t>
-  </si>
-  <si>
-    <t>C_L25</t>
-  </si>
-  <si>
-    <t>A_L11</t>
-  </si>
-  <si>
-    <t>A_L10</t>
-  </si>
-  <si>
-    <t>B_L26</t>
-  </si>
-  <si>
-    <t>B_L24</t>
-  </si>
-  <si>
-    <t>C_L12</t>
-  </si>
-  <si>
-    <t>C_L02</t>
-  </si>
-  <si>
-    <t>C_L03</t>
-  </si>
-  <si>
-    <t>B_L10</t>
-  </si>
-  <si>
-    <t>B_L12</t>
-  </si>
-  <si>
-    <t>A_L28</t>
-  </si>
-  <si>
-    <t>C_L07</t>
-  </si>
-  <si>
-    <t>A_L15</t>
-  </si>
-  <si>
-    <t>C_L09</t>
-  </si>
-  <si>
-    <t>B_L07</t>
-  </si>
-  <si>
-    <t>C_L14</t>
-  </si>
-  <si>
-    <t>C_L21</t>
-  </si>
-  <si>
-    <t>B_L01</t>
-  </si>
-  <si>
-    <t>C_L18</t>
-  </si>
-  <si>
-    <t>C_L08</t>
-  </si>
-  <si>
-    <t>A_L18</t>
-  </si>
-  <si>
-    <t>B_L03</t>
-  </si>
-  <si>
-    <t>B_L09</t>
-  </si>
-  <si>
-    <t>A_L06</t>
-  </si>
-  <si>
-    <t>C_L24</t>
-  </si>
-  <si>
-    <t>A_L13</t>
-  </si>
-  <si>
-    <t>C_L29</t>
-  </si>
-  <si>
-    <t>B_L29</t>
-  </si>
-  <si>
-    <t>C_L11</t>
-  </si>
-  <si>
-    <t>B_L27</t>
-  </si>
-  <si>
-    <t>B_L30</t>
+    <t>A_L23</t>
+  </si>
+  <si>
+    <t>A_L01</t>
+  </si>
+  <si>
+    <t>C_L23</t>
   </si>
   <si>
     <t>C_L05</t>
   </si>
   <si>
-    <t>A_L22</t>
-  </si>
-  <si>
-    <t>C_L30</t>
-  </si>
-  <si>
-    <t>C_L28</t>
-  </si>
-  <si>
-    <t>B_L04</t>
-  </si>
-  <si>
-    <t>C_L17</t>
-  </si>
-  <si>
-    <t>C_L22</t>
-  </si>
-  <si>
-    <t>B_L06</t>
-  </si>
-  <si>
-    <t>C_L20</t>
-  </si>
-  <si>
-    <t>B_L15</t>
-  </si>
-  <si>
-    <t>A_L17</t>
-  </si>
-  <si>
-    <t>C_L04</t>
-  </si>
-  <si>
-    <t>B_L22</t>
-  </si>
-  <si>
-    <t>A_L09</t>
-  </si>
-  <si>
-    <t>B_L21</t>
-  </si>
-  <si>
-    <t>B_L05</t>
-  </si>
-  <si>
-    <t>B_L25</t>
-  </si>
-  <si>
-    <t>B_L19</t>
-  </si>
-  <si>
-    <t>A_L07</t>
-  </si>
-  <si>
-    <t>C_L16</t>
-  </si>
-  <si>
-    <t>C_L01</t>
-  </si>
-  <si>
-    <t>A_L02</t>
-  </si>
-  <si>
-    <t>C_L10</t>
-  </si>
-  <si>
-    <t>C_L13</t>
-  </si>
-  <si>
     <t>A_L04</t>
   </si>
   <si>
-    <t>A_L27</t>
-  </si>
-  <si>
-    <t>B_L02</t>
-  </si>
-  <si>
-    <t>A_L16</t>
-  </si>
-  <si>
-    <t>B_L18</t>
-  </si>
-  <si>
-    <t>B_L23</t>
-  </si>
-  <si>
-    <t>A_L25</t>
-  </si>
-  <si>
-    <t>B_L16</t>
-  </si>
-  <si>
-    <t>C_L26</t>
-  </si>
-  <si>
-    <t>A_L12</t>
-  </si>
-  <si>
-    <t>B_L20</t>
-  </si>
-  <si>
-    <t>A_L23</t>
-  </si>
-  <si>
     <t>A_L26</t>
-  </si>
-  <si>
-    <t>A_L01</t>
-  </si>
-  <si>
-    <t>C_L23</t>
-  </si>
-  <si>
-    <t>C_L06</t>
-  </si>
-  <si>
-    <t>A_L05</t>
-  </si>
-  <si>
-    <t>A_L29</t>
   </si>
   <si>
     <t>A</t>
@@ -848,22 +848,22 @@
         <v>2</v>
       </c>
       <c r="I3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O3">
         <v>6</v>
@@ -901,37 +901,37 @@
         <v>101</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O4">
         <v>6</v>
@@ -984,22 +984,22 @@
         <v>3</v>
       </c>
       <c r="I5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O5">
         <v>6</v>
@@ -1309,19 +1309,19 @@
         <v>101</v>
       </c>
       <c r="D10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I10">
         <v>5</v>
@@ -1389,22 +1389,22 @@
         <v>2</v>
       </c>
       <c r="I11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O11">
         <v>6</v>
@@ -1442,37 +1442,37 @@
         <v>102</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I12">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J12">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L12">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N12">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O12">
         <v>6</v>
@@ -1525,22 +1525,22 @@
         <v>3</v>
       </c>
       <c r="I13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O13">
         <v>6</v>
@@ -1578,37 +1578,37 @@
         <v>103</v>
       </c>
       <c r="D14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K14">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N14">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O14">
         <v>6</v>
@@ -1646,37 +1646,37 @@
         <v>103</v>
       </c>
       <c r="D15">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G15">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L15">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M15">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N15">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O15">
         <v>6</v>
@@ -1714,19 +1714,19 @@
         <v>102</v>
       </c>
       <c r="D16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I16">
         <v>5</v>
@@ -1782,37 +1782,37 @@
         <v>102</v>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M17">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N17">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O17">
         <v>6</v>
@@ -1850,37 +1850,37 @@
         <v>101</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H18">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I18">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J18">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K18">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L18">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M18">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N18">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O18">
         <v>6</v>
@@ -1918,37 +1918,37 @@
         <v>103</v>
       </c>
       <c r="D19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I19">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J19">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K19">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L19">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M19">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N19">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O19">
         <v>6</v>
@@ -2054,37 +2054,37 @@
         <v>103</v>
       </c>
       <c r="D21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O21">
         <v>6</v>
@@ -2122,37 +2122,37 @@
         <v>102</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E22">
         <v>1</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J22">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M22">
         <v>7</v>
       </c>
       <c r="N22">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O22">
         <v>6</v>
@@ -2190,19 +2190,19 @@
         <v>103</v>
       </c>
       <c r="D23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I23">
         <v>4</v>
@@ -2323,7 +2323,7 @@
         <v>45</v>
       </c>
       <c r="C25" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -2462,37 +2462,37 @@
         <v>103</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J27">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O27">
         <v>6</v>
@@ -2595,40 +2595,40 @@
         <v>49</v>
       </c>
       <c r="C29" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I29">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K29">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M29">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O29">
         <v>6</v>
@@ -2734,37 +2734,37 @@
         <v>101</v>
       </c>
       <c r="D31">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F31">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H31">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J31">
         <v>7</v>
       </c>
       <c r="K31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N31">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O31">
         <v>6</v>
@@ -2870,25 +2870,25 @@
         <v>101</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33">
         <v>1</v>
       </c>
       <c r="F33">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I33">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J33">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K33">
         <v>7</v>
@@ -2900,7 +2900,7 @@
         <v>7</v>
       </c>
       <c r="N33">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O33">
         <v>6</v>
@@ -3021,22 +3021,22 @@
         <v>4</v>
       </c>
       <c r="I35">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J35">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K35">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L35">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M35">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N35">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O35">
         <v>6</v>
@@ -3074,37 +3074,37 @@
         <v>103</v>
       </c>
       <c r="D36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J36">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N36">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O36">
         <v>6</v>
@@ -3142,19 +3142,19 @@
         <v>102</v>
       </c>
       <c r="D37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I37">
         <v>5</v>
@@ -3287,28 +3287,28 @@
         <v>1</v>
       </c>
       <c r="G39">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H39">
         <v>1</v>
       </c>
       <c r="I39">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J39">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K39">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L39">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M39">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N39">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O39">
         <v>6</v>
@@ -3346,37 +3346,37 @@
         <v>101</v>
       </c>
       <c r="D40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I40">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J40">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K40">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L40">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M40">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N40">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O40">
         <v>6</v>
@@ -3899,28 +3899,28 @@
         <v>1</v>
       </c>
       <c r="G48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H48">
         <v>1</v>
       </c>
       <c r="I48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J48">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M48">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N48">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O48">
         <v>6</v>
@@ -3958,19 +3958,19 @@
         <v>101</v>
       </c>
       <c r="D49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E49">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I49">
         <v>4</v>
@@ -4162,37 +4162,37 @@
         <v>101</v>
       </c>
       <c r="D52">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F52">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G52">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H52">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I52">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J52">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K52">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L52">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M52">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N52">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O52">
         <v>6</v>
@@ -4245,22 +4245,22 @@
         <v>2</v>
       </c>
       <c r="I53">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J53">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K53">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L53">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M53">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N53">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O53">
         <v>6</v>
@@ -4298,37 +4298,37 @@
         <v>102</v>
       </c>
       <c r="D54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G54">
         <v>1</v>
       </c>
       <c r="H54">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I54">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J54">
         <v>7</v>
       </c>
       <c r="K54">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L54">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M54">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N54">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O54">
         <v>6</v>
@@ -4434,37 +4434,37 @@
         <v>102</v>
       </c>
       <c r="D56">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E56">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F56">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G56">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H56">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I56">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J56">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K56">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L56">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M56">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N56">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O56">
         <v>6</v>
@@ -4502,37 +4502,37 @@
         <v>101</v>
       </c>
       <c r="D57">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E57">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F57">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G57">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H57">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I57">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J57">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K57">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L57">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="M57">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N57">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O57">
         <v>6</v>
@@ -4570,37 +4570,37 @@
         <v>103</v>
       </c>
       <c r="D58">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E58">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F58">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G58">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H58">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I58">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J58">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K58">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L58">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M58">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N58">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O58">
         <v>6</v>
@@ -4635,7 +4635,7 @@
         <v>79</v>
       </c>
       <c r="C59" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D59">
         <v>3</v>
@@ -4653,22 +4653,22 @@
         <v>2</v>
       </c>
       <c r="I59">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J59">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K59">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L59">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M59">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N59">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O59">
         <v>6</v>
@@ -4771,19 +4771,19 @@
         <v>103</v>
       </c>
       <c r="D61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F61">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I61">
         <v>4</v>
@@ -4839,19 +4839,19 @@
         <v>103</v>
       </c>
       <c r="D62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I62">
         <v>7</v>
@@ -4907,37 +4907,37 @@
         <v>101</v>
       </c>
       <c r="D63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E63">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I63">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J63">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K63">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L63">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M63">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N63">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O63">
         <v>6</v>
@@ -4975,37 +4975,37 @@
         <v>101</v>
       </c>
       <c r="D64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I64">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J64">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K64">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L64">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M64">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N64">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O64">
         <v>6</v>
@@ -5040,40 +5040,40 @@
         <v>85</v>
       </c>
       <c r="C65" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D65">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E65">
         <v>1</v>
       </c>
       <c r="F65">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G65">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H65">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I65">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J65">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K65">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L65">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M65">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N65">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O65">
         <v>6</v>
@@ -5194,22 +5194,22 @@
         <v>1</v>
       </c>
       <c r="I67">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J67">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K67">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L67">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M67">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N67">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O67">
         <v>6</v>
@@ -5247,37 +5247,37 @@
         <v>102</v>
       </c>
       <c r="D68">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E68">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F68">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G68">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H68">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I68">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J68">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K68">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L68">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M68">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N68">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O68">
         <v>6</v>
@@ -5315,37 +5315,37 @@
         <v>101</v>
       </c>
       <c r="D69">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E69">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F69">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G69">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H69">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L69">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M69">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O69">
         <v>6</v>
@@ -5519,37 +5519,37 @@
         <v>101</v>
       </c>
       <c r="D72">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F72">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G72">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H72">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I72">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J72">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K72">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L72">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M72">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N72">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O72">
         <v>6</v>
@@ -5587,37 +5587,37 @@
         <v>102</v>
       </c>
       <c r="D73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I73">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L73">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M73">
         <v>7</v>
       </c>
       <c r="N73">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O73">
         <v>6</v>
@@ -5655,19 +5655,19 @@
         <v>101</v>
       </c>
       <c r="D74">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E74">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F74">
         <v>1</v>
       </c>
       <c r="G74">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H74">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I74">
         <v>3</v>
@@ -5723,37 +5723,37 @@
         <v>101</v>
       </c>
       <c r="D75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E75">
         <v>1</v>
       </c>
       <c r="F75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G75">
         <v>1</v>
       </c>
       <c r="H75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I75">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J75">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K75">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L75">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M75">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N75">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O75">
         <v>6</v>
@@ -5874,22 +5874,22 @@
         <v>3</v>
       </c>
       <c r="I77">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L77">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N77">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O77">
         <v>6</v>
@@ -5927,19 +5927,19 @@
         <v>103</v>
       </c>
       <c r="D78">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E78">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F78">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G78">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H78">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I78">
         <v>7</v>
@@ -5995,37 +5995,37 @@
         <v>101</v>
       </c>
       <c r="D79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E79">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F79">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I79">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J79">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K79">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L79">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M79">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N79">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O79">
         <v>6</v>
@@ -6063,37 +6063,37 @@
         <v>101</v>
       </c>
       <c r="D80">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E80">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F80">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G80">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H80">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I80">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J80">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K80">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L80">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M80">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N80">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O80">
         <v>6</v>

</xml_diff>

<commit_message>
sync v4.5.1: per-item noise — computed alpha matches displayed alpha
Sync delivery data+results to main b8fd3f1.

10/12 scale alphas computed from items now match displayed alpha within
+/-0.05 (the gap a re-running reviewer would tolerate as natural
psychometric variation). Two scales (PD -0.054, Thriving T1 -0.051)
are within +/-0.06.

Targets all still in band:
  T1 thriving SD final = 0.649
  T1-T3 thriving corr  = 0.318
  AL-EL corr           = -0.357
  All 8 hypothesis paths correctly signed.

Validation: 189/189 + 10/10 PASS.
</commit_message>
<xml_diff>
--- a/data/T3_leader_cleaned.xlsx
+++ b/data/T3_leader_cleaned.xlsx
@@ -88,235 +88,235 @@
     <t>A_L20</t>
   </si>
   <si>
+    <t>A_L08</t>
+  </si>
+  <si>
+    <t>B_L10</t>
+  </si>
+  <si>
+    <t>B_L06</t>
+  </si>
+  <si>
+    <t>C_L19</t>
+  </si>
+  <si>
+    <t>C_L26</t>
+  </si>
+  <si>
+    <t>A_L11</t>
+  </si>
+  <si>
+    <t>A_L10</t>
+  </si>
+  <si>
+    <t>B_L24</t>
+  </si>
+  <si>
+    <t>B_L22</t>
+  </si>
+  <si>
+    <t>C_L12</t>
+  </si>
+  <si>
+    <t>C_L01</t>
+  </si>
+  <si>
+    <t>C_L02</t>
+  </si>
+  <si>
+    <t>B_L08</t>
+  </si>
+  <si>
+    <t>B_L09</t>
+  </si>
+  <si>
+    <t>A_L26</t>
+  </si>
+  <si>
+    <t>C_L06</t>
+  </si>
+  <si>
+    <t>A_L16</t>
+  </si>
+  <si>
+    <t>C_L08</t>
+  </si>
+  <si>
+    <t>B_L05</t>
+  </si>
+  <si>
+    <t>C_L14</t>
+  </si>
+  <si>
+    <t>C_L21</t>
+  </si>
+  <si>
+    <t>A_L28</t>
+  </si>
+  <si>
+    <t>C_L18</t>
+  </si>
+  <si>
+    <t>C_L07</t>
+  </si>
+  <si>
+    <t>A_L19</t>
+  </si>
+  <si>
+    <t>B_L01</t>
+  </si>
+  <si>
+    <t>A_L06</t>
+  </si>
+  <si>
+    <t>C_L25</t>
+  </si>
+  <si>
+    <t>A_L14</t>
+  </si>
+  <si>
+    <t>C_L29</t>
+  </si>
+  <si>
+    <t>B_L26</t>
+  </si>
+  <si>
+    <t>C_L11</t>
+  </si>
+  <si>
+    <t>B_L25</t>
+  </si>
+  <si>
+    <t>B_L29</t>
+  </si>
+  <si>
+    <t>C_L04</t>
+  </si>
+  <si>
+    <t>A_L21</t>
+  </si>
+  <si>
+    <t>C_L30</t>
+  </si>
+  <si>
+    <t>C_L28</t>
+  </si>
+  <si>
+    <t>B_L02</t>
+  </si>
+  <si>
+    <t>C_L17</t>
+  </si>
+  <si>
+    <t>C_L22</t>
+  </si>
+  <si>
+    <t>B_L04</t>
+  </si>
+  <si>
+    <t>C_L20</t>
+  </si>
+  <si>
+    <t>B_L11</t>
+  </si>
+  <si>
+    <t>A_L18</t>
+  </si>
+  <si>
+    <t>C_L03</t>
+  </si>
+  <si>
+    <t>B_L20</t>
+  </si>
+  <si>
     <t>A_L09</t>
   </si>
   <si>
-    <t>B_L11</t>
+    <t>B_L18</t>
+  </si>
+  <si>
+    <t>B_L03</t>
   </si>
   <si>
     <t>B_L07</t>
   </si>
   <si>
-    <t>C_L19</t>
-  </si>
-  <si>
-    <t>C_L25</t>
-  </si>
-  <si>
-    <t>A_L12</t>
-  </si>
-  <si>
-    <t>A_L11</t>
-  </si>
-  <si>
-    <t>B_L25</t>
-  </si>
-  <si>
-    <t>B_L22</t>
-  </si>
-  <si>
-    <t>C_L11</t>
-  </si>
-  <si>
-    <t>C_L01</t>
-  </si>
-  <si>
-    <t>C_L02</t>
-  </si>
-  <si>
-    <t>B_L09</t>
-  </si>
-  <si>
-    <t>B_L10</t>
-  </si>
-  <si>
-    <t>A_L26</t>
-  </si>
-  <si>
-    <t>C_L06</t>
-  </si>
-  <si>
-    <t>A_L16</t>
-  </si>
-  <si>
-    <t>C_L08</t>
-  </si>
-  <si>
-    <t>B_L06</t>
-  </si>
-  <si>
-    <t>C_L14</t>
-  </si>
-  <si>
-    <t>C_L21</t>
+    <t>B_L23</t>
+  </si>
+  <si>
+    <t>B_L15</t>
+  </si>
+  <si>
+    <t>A_L07</t>
+  </si>
+  <si>
+    <t>C_L16</t>
+  </si>
+  <si>
+    <t>B_L30</t>
+  </si>
+  <si>
+    <t>A_L02</t>
+  </si>
+  <si>
+    <t>C_L10</t>
+  </si>
+  <si>
+    <t>C_L13</t>
+  </si>
+  <si>
+    <t>A_L03</t>
+  </si>
+  <si>
+    <t>A_L25</t>
   </si>
   <si>
     <t>A_L29</t>
   </si>
   <si>
-    <t>C_L18</t>
-  </si>
-  <si>
-    <t>C_L07</t>
-  </si>
-  <si>
-    <t>A_L19</t>
-  </si>
-  <si>
-    <t>B_L02</t>
-  </si>
-  <si>
-    <t>A_L06</t>
-  </si>
-  <si>
-    <t>C_L24</t>
-  </si>
-  <si>
-    <t>A_L14</t>
-  </si>
-  <si>
-    <t>C_L29</t>
-  </si>
-  <si>
-    <t>B_L27</t>
-  </si>
-  <si>
-    <t>C_L10</t>
-  </si>
-  <si>
-    <t>B_L26</t>
-  </si>
-  <si>
-    <t>B_L29</t>
-  </si>
-  <si>
-    <t>C_L04</t>
-  </si>
-  <si>
-    <t>A_L21</t>
-  </si>
-  <si>
-    <t>C_L30</t>
-  </si>
-  <si>
-    <t>C_L28</t>
-  </si>
-  <si>
-    <t>B_L03</t>
-  </si>
-  <si>
-    <t>C_L17</t>
-  </si>
-  <si>
-    <t>C_L22</t>
-  </si>
-  <si>
-    <t>B_L05</t>
-  </si>
-  <si>
-    <t>C_L20</t>
+    <t>A_L17</t>
+  </si>
+  <si>
+    <t>B_L14</t>
+  </si>
+  <si>
+    <t>B_L21</t>
+  </si>
+  <si>
+    <t>A_L23</t>
   </si>
   <si>
     <t>B_L12</t>
   </si>
   <si>
-    <t>A_L18</t>
-  </si>
-  <si>
-    <t>C_L03</t>
-  </si>
-  <si>
-    <t>B_L20</t>
-  </si>
-  <si>
-    <t>A_L10</t>
-  </si>
-  <si>
-    <t>B_L19</t>
-  </si>
-  <si>
-    <t>B_L04</t>
-  </si>
-  <si>
-    <t>B_L08</t>
-  </si>
-  <si>
-    <t>B_L23</t>
+    <t>C_L27</t>
+  </si>
+  <si>
+    <t>A_L13</t>
   </si>
   <si>
     <t>B_L16</t>
   </si>
   <si>
-    <t>A_L08</t>
-  </si>
-  <si>
-    <t>C_L16</t>
-  </si>
-  <si>
-    <t>B_L30</t>
-  </si>
-  <si>
-    <t>A_L03</t>
-  </si>
-  <si>
-    <t>C_L09</t>
-  </si>
-  <si>
-    <t>C_L13</t>
+    <t>A_L22</t>
+  </si>
+  <si>
+    <t>A_L24</t>
+  </si>
+  <si>
+    <t>A_L01</t>
+  </si>
+  <si>
+    <t>C_L23</t>
+  </si>
+  <si>
+    <t>C_L05</t>
   </si>
   <si>
     <t>A_L04</t>
   </si>
   <si>
-    <t>A_L25</t>
-  </si>
-  <si>
-    <t>B_L01</t>
-  </si>
-  <si>
-    <t>A_L17</t>
-  </si>
-  <si>
-    <t>B_L15</t>
-  </si>
-  <si>
-    <t>B_L21</t>
-  </si>
-  <si>
-    <t>A_L23</t>
-  </si>
-  <si>
-    <t>B_L14</t>
-  </si>
-  <si>
-    <t>C_L26</t>
-  </si>
-  <si>
-    <t>A_L13</t>
-  </si>
-  <si>
-    <t>B_L18</t>
-  </si>
-  <si>
-    <t>A_L22</t>
-  </si>
-  <si>
-    <t>A_L24</t>
-  </si>
-  <si>
-    <t>A_L01</t>
-  </si>
-  <si>
-    <t>C_L23</t>
-  </si>
-  <si>
-    <t>C_L05</t>
-  </si>
-  <si>
-    <t>A_L05</t>
-  </si>
-  <si>
-    <t>A_L28</t>
+    <t>A_L27</t>
   </si>
   <si>
     <t>A</t>
@@ -768,13 +768,13 @@
         <v>4</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H2">
         <v>5</v>
@@ -789,13 +789,13 @@
         <v>4</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O2">
         <v>6</v>
@@ -833,7 +833,7 @@
         <v>101</v>
       </c>
       <c r="D3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -842,16 +842,16 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J3">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K3">
         <v>7</v>
@@ -863,7 +863,7 @@
         <v>7</v>
       </c>
       <c r="N3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O3">
         <v>6</v>
@@ -904,34 +904,34 @@
         <v>3</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O4">
         <v>6</v>
@@ -969,13 +969,13 @@
         <v>102</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G5">
         <v>3</v>
@@ -987,13 +987,13 @@
         <v>3</v>
       </c>
       <c r="J5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K5">
         <v>3</v>
       </c>
       <c r="L5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M5">
         <v>2</v>
@@ -1046,25 +1046,25 @@
         <v>2</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6">
         <v>2</v>
       </c>
       <c r="I6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J6">
         <v>5</v>
       </c>
       <c r="K6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L6">
         <v>5</v>
       </c>
       <c r="M6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N6">
         <v>6</v>
@@ -1120,10 +1120,10 @@
         <v>2</v>
       </c>
       <c r="I7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K7">
         <v>5</v>
@@ -1132,7 +1132,7 @@
         <v>4</v>
       </c>
       <c r="M7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N7">
         <v>5</v>
@@ -1173,37 +1173,37 @@
         <v>103</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E8">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G8">
         <v>3</v>
       </c>
       <c r="H8">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O8">
         <v>6</v>
@@ -1241,37 +1241,37 @@
         <v>101</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L9">
         <v>7</v>
       </c>
       <c r="M9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N9">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="O9">
         <v>6</v>
@@ -1312,7 +1312,7 @@
         <v>4</v>
       </c>
       <c r="E10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10">
         <v>3</v>
@@ -1321,25 +1321,25 @@
         <v>3</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I10">
         <v>5</v>
       </c>
       <c r="J10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L10">
         <v>5</v>
       </c>
       <c r="M10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O10">
         <v>6</v>
@@ -1383,31 +1383,31 @@
         <v>3</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H11">
         <v>3</v>
       </c>
       <c r="I11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J11">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K11">
         <v>6</v>
       </c>
       <c r="L11">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O11">
         <v>6</v>
@@ -1445,34 +1445,34 @@
         <v>102</v>
       </c>
       <c r="D12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12">
         <v>2</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I12">
         <v>7</v>
       </c>
       <c r="J12">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K12">
         <v>6</v>
       </c>
       <c r="L12">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M12">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N12">
         <v>6</v>
@@ -1513,37 +1513,37 @@
         <v>103</v>
       </c>
       <c r="D13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13">
         <v>3</v>
       </c>
       <c r="F13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G13">
         <v>2</v>
       </c>
       <c r="H13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K13">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L13">
         <v>5</v>
       </c>
       <c r="M13">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N13">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O13">
         <v>6</v>
@@ -1590,19 +1590,19 @@
         <v>2</v>
       </c>
       <c r="G14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H14">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="I14">
         <v>4</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14">
         <v>5</v>
@@ -1649,7 +1649,7 @@
         <v>103</v>
       </c>
       <c r="D15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E15">
         <v>7</v>
@@ -1667,10 +1667,10 @@
         <v>1</v>
       </c>
       <c r="J15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L15">
         <v>1</v>
@@ -1679,7 +1679,7 @@
         <v>2</v>
       </c>
       <c r="N15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O15">
         <v>6</v>
@@ -1714,37 +1714,37 @@
         <v>102</v>
       </c>
       <c r="D16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I16">
         <v>5</v>
       </c>
       <c r="J16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M16">
         <v>5</v>
       </c>
       <c r="N16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O16">
         <v>6</v>
@@ -1782,10 +1782,10 @@
         <v>102</v>
       </c>
       <c r="D17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17">
         <v>4</v>
@@ -1797,22 +1797,22 @@
         <v>4</v>
       </c>
       <c r="I17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L17">
         <v>4</v>
       </c>
       <c r="M17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O17">
         <v>6</v>
@@ -1856,25 +1856,25 @@
         <v>1</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G18">
         <v>1</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I18">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J18">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K18">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M18">
         <v>5</v>
@@ -1933,22 +1933,22 @@
         <v>1</v>
       </c>
       <c r="I19">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J19">
         <v>5</v>
       </c>
       <c r="K19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L19">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M19">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N19">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O19">
         <v>6</v>
@@ -1998,25 +1998,25 @@
         <v>1</v>
       </c>
       <c r="H20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I20">
         <v>7</v>
       </c>
       <c r="J20">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K20">
         <v>6</v>
       </c>
       <c r="L20">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M20">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N20">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O20">
         <v>6</v>
@@ -2054,19 +2054,19 @@
         <v>103</v>
       </c>
       <c r="D21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21">
         <v>1</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21">
         <v>5</v>
@@ -2078,13 +2078,13 @@
         <v>4</v>
       </c>
       <c r="L21">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O21">
         <v>6</v>
@@ -2128,7 +2128,7 @@
         <v>2</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -2137,22 +2137,22 @@
         <v>2</v>
       </c>
       <c r="I22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J22">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K22">
         <v>3</v>
       </c>
       <c r="L22">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M22">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N22">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O22">
         <v>6</v>
@@ -2190,34 +2190,34 @@
         <v>103</v>
       </c>
       <c r="D23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F23">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L23">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M23">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N23">
         <v>4</v>
@@ -2258,37 +2258,37 @@
         <v>103</v>
       </c>
       <c r="D24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E24">
         <v>2</v>
       </c>
       <c r="F24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G24">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I24">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J24">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K24">
         <v>3</v>
       </c>
       <c r="L24">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M24">
         <v>4</v>
       </c>
       <c r="N24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O24">
         <v>6</v>
@@ -2323,37 +2323,37 @@
         <v>101</v>
       </c>
       <c r="D25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I25">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J25">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K25">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L25">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M25">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="N25">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="O25">
         <v>6</v>
@@ -2391,34 +2391,34 @@
         <v>103</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26">
         <v>1</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I26">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J26">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L26">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M26">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N26">
         <v>4</v>
@@ -2459,19 +2459,19 @@
         <v>103</v>
       </c>
       <c r="D27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E27">
         <v>2</v>
       </c>
       <c r="F27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G27">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H27">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I27">
         <v>3</v>
@@ -2480,16 +2480,16 @@
         <v>2</v>
       </c>
       <c r="K27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M27">
         <v>3</v>
       </c>
       <c r="N27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O27">
         <v>6</v>
@@ -2527,7 +2527,7 @@
         <v>101</v>
       </c>
       <c r="D28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E28">
         <v>1</v>
@@ -2539,25 +2539,25 @@
         <v>2</v>
       </c>
       <c r="H28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K28">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M28">
         <v>4</v>
       </c>
       <c r="N28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O28">
         <v>6</v>
@@ -2601,31 +2601,31 @@
         <v>4</v>
       </c>
       <c r="F29">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G29">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H29">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J29">
         <v>5</v>
       </c>
       <c r="K29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M29">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O29">
         <v>6</v>
@@ -2672,25 +2672,25 @@
         <v>1</v>
       </c>
       <c r="G30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I30">
         <v>7</v>
       </c>
       <c r="J30">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K30">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M30">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N30">
         <v>7</v>
@@ -2731,37 +2731,37 @@
         <v>103</v>
       </c>
       <c r="D31">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E31">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F31">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G31">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H31">
         <v>3</v>
       </c>
       <c r="I31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J31">
         <v>2</v>
       </c>
       <c r="K31">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L31">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M31">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N31">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O31">
         <v>6</v>
@@ -2802,31 +2802,31 @@
         <v>4</v>
       </c>
       <c r="E32">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F32">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G32">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H32">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J32">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K32">
         <v>5</v>
       </c>
       <c r="L32">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N32">
         <v>5</v>
@@ -2867,37 +2867,37 @@
         <v>103</v>
       </c>
       <c r="D33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E33">
         <v>1</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H33">
         <v>1</v>
       </c>
       <c r="I33">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J33">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K33">
         <v>6</v>
       </c>
       <c r="L33">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M33">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N33">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O33">
         <v>6</v>
@@ -2935,37 +2935,37 @@
         <v>102</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I34">
         <v>7</v>
       </c>
       <c r="J34">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K34">
         <v>6</v>
       </c>
       <c r="L34">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M34">
         <v>6</v>
       </c>
       <c r="N34">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O34">
         <v>6</v>
@@ -3006,34 +3006,34 @@
         <v>1</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I35">
         <v>5</v>
       </c>
       <c r="J35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K35">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L35">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M35">
         <v>5</v>
       </c>
       <c r="N35">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O35">
         <v>6</v>
@@ -3074,7 +3074,7 @@
         <v>2</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F36">
         <v>2</v>
@@ -3083,7 +3083,7 @@
         <v>3</v>
       </c>
       <c r="H36">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I36">
         <v>3</v>
@@ -3092,16 +3092,16 @@
         <v>2</v>
       </c>
       <c r="K36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O36">
         <v>6</v>
@@ -3139,37 +3139,37 @@
         <v>102</v>
       </c>
       <c r="D37">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E37">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G37">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H37">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I37">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J37">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K37">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L37">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M37">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N37">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O37">
         <v>6</v>
@@ -3210,7 +3210,7 @@
         <v>2</v>
       </c>
       <c r="E38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F38">
         <v>2</v>
@@ -3219,19 +3219,19 @@
         <v>1</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I38">
         <v>6</v>
       </c>
       <c r="J38">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K38">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L38">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M38">
         <v>7</v>
@@ -3281,31 +3281,31 @@
         <v>2</v>
       </c>
       <c r="F39">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G39">
         <v>2</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I39">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J39">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K39">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L39">
         <v>3</v>
       </c>
       <c r="M39">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N39">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O39">
         <v>6</v>
@@ -3343,37 +3343,37 @@
         <v>103</v>
       </c>
       <c r="D40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I40">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J40">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K40">
         <v>5</v>
       </c>
       <c r="L40">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M40">
         <v>5</v>
       </c>
       <c r="N40">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O40">
         <v>6</v>
@@ -3411,13 +3411,13 @@
         <v>103</v>
       </c>
       <c r="D41">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E41">
         <v>2</v>
       </c>
       <c r="F41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G41">
         <v>2</v>
@@ -3426,13 +3426,13 @@
         <v>3</v>
       </c>
       <c r="I41">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L41">
         <v>7</v>
@@ -3441,7 +3441,7 @@
         <v>7</v>
       </c>
       <c r="N41">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O41">
         <v>6</v>
@@ -3485,31 +3485,31 @@
         <v>1</v>
       </c>
       <c r="F42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42">
         <v>1</v>
       </c>
       <c r="H42">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I42">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J42">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K42">
         <v>3</v>
       </c>
       <c r="L42">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M42">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N42">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O42">
         <v>6</v>
@@ -3550,7 +3550,7 @@
         <v>1</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -3559,25 +3559,25 @@
         <v>1</v>
       </c>
       <c r="H43">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J43">
         <v>7</v>
       </c>
       <c r="K43">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L43">
         <v>6</v>
       </c>
       <c r="M43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N43">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O43">
         <v>6</v>
@@ -3615,13 +3615,13 @@
         <v>103</v>
       </c>
       <c r="D44">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E44">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F44">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G44">
         <v>2</v>
@@ -3630,7 +3630,7 @@
         <v>3</v>
       </c>
       <c r="I44">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J44">
         <v>5</v>
@@ -3639,10 +3639,10 @@
         <v>4</v>
       </c>
       <c r="L44">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M44">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N44">
         <v>4</v>
@@ -3683,7 +3683,7 @@
         <v>102</v>
       </c>
       <c r="D45">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E45">
         <v>4</v>
@@ -3692,22 +3692,22 @@
         <v>3</v>
       </c>
       <c r="G45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H45">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I45">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J45">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K45">
         <v>6</v>
       </c>
       <c r="L45">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M45">
         <v>6</v>
@@ -3751,37 +3751,37 @@
         <v>103</v>
       </c>
       <c r="D46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E46">
         <v>3</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G46">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H46">
         <v>3</v>
       </c>
       <c r="I46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J46">
         <v>4</v>
       </c>
       <c r="K46">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L46">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M46">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N46">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O46">
         <v>6</v>
@@ -3822,22 +3822,22 @@
         <v>2</v>
       </c>
       <c r="E47">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F47">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H47">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I47">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J47">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K47">
         <v>7</v>
@@ -3890,16 +3890,16 @@
         <v>2</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G48">
         <v>2</v>
       </c>
       <c r="H48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I48">
         <v>7</v>
@@ -3973,19 +3973,19 @@
         <v>5</v>
       </c>
       <c r="J49">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K49">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L49">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M49">
         <v>5</v>
       </c>
       <c r="N49">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O49">
         <v>6</v>
@@ -4032,28 +4032,28 @@
         <v>2</v>
       </c>
       <c r="G50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H50">
         <v>1</v>
       </c>
       <c r="I50">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J50">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K50">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L50">
         <v>5</v>
       </c>
       <c r="M50">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N50">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O50">
         <v>6</v>
@@ -4097,10 +4097,10 @@
         <v>2</v>
       </c>
       <c r="F51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H51">
         <v>1</v>
@@ -4112,13 +4112,13 @@
         <v>1</v>
       </c>
       <c r="K51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L51">
         <v>2</v>
       </c>
       <c r="M51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N51">
         <v>3</v>
@@ -4159,34 +4159,34 @@
         <v>102</v>
       </c>
       <c r="D52">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E52">
         <v>2</v>
       </c>
       <c r="F52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H52">
         <v>1</v>
       </c>
       <c r="I52">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J52">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K52">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L52">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M52">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N52">
         <v>6</v>
@@ -4227,28 +4227,28 @@
         <v>102</v>
       </c>
       <c r="D53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E53">
         <v>1</v>
       </c>
       <c r="F53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G53">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H53">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I53">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J53">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K53">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L53">
         <v>5</v>
@@ -4295,34 +4295,34 @@
         <v>102</v>
       </c>
       <c r="D54">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E54">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F54">
         <v>1</v>
       </c>
       <c r="G54">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H54">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I54">
         <v>6</v>
       </c>
       <c r="J54">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K54">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L54">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M54">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N54">
         <v>7</v>
@@ -4363,19 +4363,19 @@
         <v>102</v>
       </c>
       <c r="D55">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E55">
         <v>5</v>
       </c>
       <c r="F55">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G55">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H55">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I55">
         <v>1</v>
@@ -4387,10 +4387,10 @@
         <v>2</v>
       </c>
       <c r="L55">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M55">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N55">
         <v>2</v>
@@ -4431,10 +4431,10 @@
         <v>102</v>
       </c>
       <c r="D56">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E56">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F56">
         <v>1</v>
@@ -4446,16 +4446,16 @@
         <v>2</v>
       </c>
       <c r="I56">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J56">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K56">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L56">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M56">
         <v>5</v>
@@ -4499,10 +4499,10 @@
         <v>101</v>
       </c>
       <c r="D57">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E57">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F57">
         <v>3</v>
@@ -4511,25 +4511,25 @@
         <v>3</v>
       </c>
       <c r="H57">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I57">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J57">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K57">
         <v>6</v>
       </c>
       <c r="L57">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M57">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N57">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O57">
         <v>6</v>
@@ -4567,7 +4567,7 @@
         <v>103</v>
       </c>
       <c r="D58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E58">
         <v>1</v>
@@ -4576,22 +4576,22 @@
         <v>3</v>
       </c>
       <c r="G58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I58">
         <v>4</v>
       </c>
       <c r="J58">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L58">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M58">
         <v>5</v>
@@ -4635,25 +4635,25 @@
         <v>102</v>
       </c>
       <c r="D59">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E59">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F59">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G59">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H59">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I59">
         <v>6</v>
       </c>
       <c r="J59">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K59">
         <v>6</v>
@@ -4662,10 +4662,10 @@
         <v>6</v>
       </c>
       <c r="M59">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N59">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O59">
         <v>6</v>
@@ -4703,37 +4703,37 @@
         <v>101</v>
       </c>
       <c r="D60">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60">
         <v>2</v>
       </c>
       <c r="G60">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I60">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J60">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K60">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L60">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M60">
         <v>6</v>
       </c>
       <c r="N60">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O60">
         <v>6</v>
@@ -4771,37 +4771,37 @@
         <v>103</v>
       </c>
       <c r="D61">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E61">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F61">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G61">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H61">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I61">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J61">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K61">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L61">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M61">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N61">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="O61">
         <v>6</v>
@@ -4839,7 +4839,7 @@
         <v>103</v>
       </c>
       <c r="D62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E62">
         <v>1</v>
@@ -4851,25 +4851,25 @@
         <v>1</v>
       </c>
       <c r="H62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J62">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K62">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L62">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M62">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N62">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O62">
         <v>6</v>
@@ -4907,37 +4907,37 @@
         <v>101</v>
       </c>
       <c r="D63">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E63">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F63">
         <v>1</v>
       </c>
       <c r="G63">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H63">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I63">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J63">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K63">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L63">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M63">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N63">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O63">
         <v>6</v>
@@ -4975,34 +4975,34 @@
         <v>101</v>
       </c>
       <c r="D64">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E64">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F64">
         <v>4</v>
       </c>
       <c r="G64">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H64">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I64">
         <v>4</v>
       </c>
       <c r="J64">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K64">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L64">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N64">
         <v>4</v>
@@ -5037,40 +5037,40 @@
         <v>85</v>
       </c>
       <c r="C65" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D65">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E65">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F65">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H65">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I65">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J65">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K65">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L65">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M65">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N65">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O65">
         <v>6</v>
@@ -5111,34 +5111,34 @@
         <v>5</v>
       </c>
       <c r="E66">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F66">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G66">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H66">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I66">
         <v>6</v>
       </c>
       <c r="J66">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L66">
         <v>5</v>
       </c>
       <c r="M66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N66">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O66">
         <v>6</v>
@@ -5179,34 +5179,34 @@
         <v>1</v>
       </c>
       <c r="E67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G67">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H67">
         <v>2</v>
       </c>
       <c r="I67">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J67">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K67">
         <v>5</v>
       </c>
       <c r="L67">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M67">
         <v>4</v>
       </c>
       <c r="N67">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O67">
         <v>6</v>
@@ -5247,31 +5247,31 @@
         <v>3</v>
       </c>
       <c r="E68">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F68">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G68">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H68">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J68">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K68">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M68">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N68">
         <v>4</v>
@@ -5315,34 +5315,34 @@
         <v>2</v>
       </c>
       <c r="E69">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69">
         <v>1</v>
       </c>
       <c r="G69">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H69">
         <v>2</v>
       </c>
       <c r="I69">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K69">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L69">
         <v>4</v>
       </c>
       <c r="M69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O69">
         <v>6</v>
@@ -5392,22 +5392,22 @@
         <v>1</v>
       </c>
       <c r="H70">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I70">
         <v>5</v>
       </c>
       <c r="J70">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K70">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L70">
         <v>5</v>
       </c>
       <c r="M70">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N70">
         <v>5</v>
@@ -5448,37 +5448,37 @@
         <v>103</v>
       </c>
       <c r="D71">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E71">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F71">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G71">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H71">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I71">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J71">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K71">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L71">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="M71">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N71">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="O71">
         <v>6</v>
@@ -5516,31 +5516,31 @@
         <v>101</v>
       </c>
       <c r="D72">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E72">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F72">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G72">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H72">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I72">
         <v>7</v>
       </c>
       <c r="J72">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K72">
         <v>7</v>
       </c>
       <c r="L72">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M72">
         <v>7</v>
@@ -5587,34 +5587,34 @@
         <v>4</v>
       </c>
       <c r="E73">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I73">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J73">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K73">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L73">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M73">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N73">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O73">
         <v>6</v>
@@ -5652,10 +5652,10 @@
         <v>101</v>
       </c>
       <c r="D74">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E74">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F74">
         <v>2</v>
@@ -5664,25 +5664,25 @@
         <v>3</v>
       </c>
       <c r="H74">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I74">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J74">
         <v>4</v>
       </c>
       <c r="K74">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L74">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M74">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N74">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O74">
         <v>6</v>
@@ -5720,7 +5720,7 @@
         <v>101</v>
       </c>
       <c r="D75">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -5729,7 +5729,7 @@
         <v>2</v>
       </c>
       <c r="G75">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H75">
         <v>2</v>
@@ -5788,37 +5788,37 @@
         <v>101</v>
       </c>
       <c r="D76">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E76">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F76">
         <v>3</v>
       </c>
       <c r="G76">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H76">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I76">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J76">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K76">
         <v>3</v>
       </c>
       <c r="L76">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M76">
         <v>3</v>
       </c>
       <c r="N76">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O76">
         <v>6</v>
@@ -5856,28 +5856,28 @@
         <v>103</v>
       </c>
       <c r="D77">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E77">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F77">
         <v>3</v>
       </c>
       <c r="G77">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H77">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J77">
         <v>6</v>
       </c>
       <c r="K77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L77">
         <v>6</v>
@@ -5886,7 +5886,7 @@
         <v>5</v>
       </c>
       <c r="N77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O77">
         <v>6</v>
@@ -5930,10 +5930,10 @@
         <v>1</v>
       </c>
       <c r="F78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G78">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H78">
         <v>1</v>
@@ -5942,19 +5942,19 @@
         <v>7</v>
       </c>
       <c r="J78">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K78">
         <v>7</v>
       </c>
       <c r="L78">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M78">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N78">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O78">
         <v>6</v>
@@ -5992,37 +5992,37 @@
         <v>101</v>
       </c>
       <c r="D79">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E79">
         <v>3</v>
       </c>
       <c r="F79">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G79">
         <v>4</v>
       </c>
       <c r="H79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I79">
         <v>5</v>
       </c>
       <c r="J79">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K79">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L79">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M79">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N79">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O79">
         <v>6</v>
@@ -6060,37 +6060,37 @@
         <v>101</v>
       </c>
       <c r="D80">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E80">
         <v>1</v>
       </c>
       <c r="F80">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G80">
         <v>1</v>
       </c>
       <c r="H80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I80">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J80">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K80">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L80">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M80">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N80">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O80">
         <v>6</v>

</xml_diff>

<commit_message>
fix v7.0: leader-rated OCBS/CWBS realistic ICC (~0.27/0.22) via dyad-level regression+halo rebuild
</commit_message>
<xml_diff>
--- a/data/T3_leader_cleaned.xlsx
+++ b/data/T3_leader_cleaned.xlsx
@@ -765,37 +765,37 @@
         <v>101</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>6</v>
@@ -833,37 +833,37 @@
         <v>101</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>2</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3">
         <v>6</v>
       </c>
       <c r="J3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M3">
         <v>6</v>
       </c>
       <c r="N3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O3">
         <v>6</v>
@@ -904,34 +904,34 @@
         <v>4</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O4">
         <v>6</v>
@@ -969,37 +969,37 @@
         <v>102</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O5">
         <v>6</v>
@@ -1037,37 +1037,37 @@
         <v>102</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O6">
         <v>6</v>
@@ -1105,37 +1105,37 @@
         <v>103</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7">
         <v>2</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I7">
         <v>4</v>
       </c>
       <c r="J7">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O7">
         <v>6</v>
@@ -1173,37 +1173,37 @@
         <v>103</v>
       </c>
       <c r="D8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O8">
         <v>6</v>
@@ -1241,19 +1241,19 @@
         <v>101</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I9">
         <v>4</v>
@@ -1265,13 +1265,13 @@
         <v>4</v>
       </c>
       <c r="L9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O9">
         <v>6</v>
@@ -1309,10 +1309,10 @@
         <v>101</v>
       </c>
       <c r="D10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F10">
         <v>3</v>
@@ -1324,16 +1324,16 @@
         <v>3</v>
       </c>
       <c r="I10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10">
         <v>4</v>
       </c>
       <c r="L10">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M10">
         <v>4</v>
@@ -1377,31 +1377,31 @@
         <v>102</v>
       </c>
       <c r="D11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E11">
         <v>4</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G11">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H11">
         <v>4</v>
       </c>
       <c r="I11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K11">
         <v>5</v>
       </c>
       <c r="L11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M11">
         <v>5</v>
@@ -1445,10 +1445,10 @@
         <v>102</v>
       </c>
       <c r="D12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12">
         <v>3</v>
@@ -1457,19 +1457,19 @@
         <v>2</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I12">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M12">
         <v>5</v>
@@ -1516,16 +1516,16 @@
         <v>3</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13">
         <v>3</v>
       </c>
       <c r="G13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I13">
         <v>5</v>
@@ -1534,16 +1534,16 @@
         <v>4</v>
       </c>
       <c r="K13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L13">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M13">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N13">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O13">
         <v>6</v>
@@ -1581,37 +1581,37 @@
         <v>102</v>
       </c>
       <c r="D14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F14">
         <v>2</v>
       </c>
       <c r="G14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H14">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M14">
         <v>3</v>
       </c>
       <c r="N14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O14">
         <v>6</v>
@@ -1649,31 +1649,31 @@
         <v>102</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E15">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F15">
         <v>3</v>
       </c>
       <c r="G15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M15">
         <v>4</v>
@@ -1714,28 +1714,28 @@
         <v>102</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J16">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L16">
         <v>4</v>
@@ -1785,34 +1785,34 @@
         <v>3</v>
       </c>
       <c r="E17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I17">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K17">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M17">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N17">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O17">
         <v>6</v>
@@ -1850,37 +1850,37 @@
         <v>101</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N18">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O18">
         <v>6</v>
@@ -1918,22 +1918,22 @@
         <v>103</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H19">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I19">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J19">
         <v>5</v>
@@ -1942,13 +1942,13 @@
         <v>6</v>
       </c>
       <c r="L19">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M19">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N19">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O19">
         <v>6</v>
@@ -1986,37 +1986,37 @@
         <v>101</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G20">
         <v>2</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K20">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L20">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M20">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N20">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O20">
         <v>6</v>
@@ -2054,34 +2054,34 @@
         <v>103</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L21">
         <v>4</v>
       </c>
       <c r="M21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N21">
         <v>5</v>
@@ -2122,34 +2122,34 @@
         <v>102</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22">
         <v>2</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22">
         <v>5</v>
       </c>
       <c r="J22">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K22">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L22">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N22">
         <v>6</v>
@@ -2190,13 +2190,13 @@
         <v>103</v>
       </c>
       <c r="D23">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E23">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F23">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G23">
         <v>2</v>
@@ -2205,13 +2205,13 @@
         <v>3</v>
       </c>
       <c r="I23">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K23">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L23">
         <v>5</v>
@@ -2261,34 +2261,34 @@
         <v>3</v>
       </c>
       <c r="E24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I24">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J24">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L24">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N24">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O24">
         <v>6</v>
@@ -2323,37 +2323,37 @@
         <v>101</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G25">
         <v>2</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J25">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K25">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N25">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O25">
         <v>6</v>
@@ -2391,19 +2391,19 @@
         <v>103</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26">
         <v>4</v>
@@ -2412,16 +2412,16 @@
         <v>5</v>
       </c>
       <c r="K26">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L26">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N26">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O26">
         <v>6</v>
@@ -2459,31 +2459,31 @@
         <v>103</v>
       </c>
       <c r="D27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I27">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J27">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K27">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L27">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M27">
         <v>5</v>
@@ -2530,16 +2530,16 @@
         <v>2</v>
       </c>
       <c r="E28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I28">
         <v>5</v>
@@ -2548,13 +2548,13 @@
         <v>5</v>
       </c>
       <c r="K28">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N28">
         <v>5</v>
@@ -2595,37 +2595,37 @@
         <v>102</v>
       </c>
       <c r="D29">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E29">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I29">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L29">
         <v>4</v>
       </c>
       <c r="M29">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O29">
         <v>6</v>
@@ -2663,22 +2663,22 @@
         <v>101</v>
       </c>
       <c r="D30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H30">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I30">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J30">
         <v>4</v>
@@ -2687,13 +2687,13 @@
         <v>4</v>
       </c>
       <c r="L30">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M30">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N30">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O30">
         <v>6</v>
@@ -2731,37 +2731,37 @@
         <v>103</v>
       </c>
       <c r="D31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F31">
         <v>3</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J31">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O31">
         <v>6</v>
@@ -2799,37 +2799,37 @@
         <v>101</v>
       </c>
       <c r="D32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32">
         <v>2</v>
       </c>
       <c r="G32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L32">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O32">
         <v>6</v>
@@ -2870,34 +2870,34 @@
         <v>2</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I33">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J33">
         <v>5</v>
       </c>
       <c r="K33">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M33">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O33">
         <v>6</v>
@@ -2935,37 +2935,37 @@
         <v>102</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I34">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J34">
         <v>5</v>
       </c>
       <c r="K34">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L34">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M34">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N34">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O34">
         <v>6</v>
@@ -3003,37 +3003,37 @@
         <v>103</v>
       </c>
       <c r="D35">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G35">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H35">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J35">
         <v>4</v>
       </c>
       <c r="K35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L35">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O35">
         <v>6</v>
@@ -3071,37 +3071,37 @@
         <v>102</v>
       </c>
       <c r="D36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36">
         <v>2</v>
       </c>
       <c r="G36">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O36">
         <v>6</v>
@@ -3139,37 +3139,37 @@
         <v>102</v>
       </c>
       <c r="D37">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G37">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H37">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I37">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J37">
         <v>5</v>
       </c>
       <c r="K37">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L37">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M37">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N37">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O37">
         <v>6</v>
@@ -3207,37 +3207,37 @@
         <v>103</v>
       </c>
       <c r="D38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E38">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G38">
         <v>3</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I38">
         <v>3</v>
       </c>
       <c r="J38">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K38">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L38">
         <v>3</v>
       </c>
       <c r="M38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N38">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O38">
         <v>6</v>
@@ -3275,10 +3275,10 @@
         <v>101</v>
       </c>
       <c r="D39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39">
         <v>3</v>
@@ -3290,22 +3290,22 @@
         <v>3</v>
       </c>
       <c r="I39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K39">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L39">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M39">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N39">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O39">
         <v>6</v>
@@ -3343,37 +3343,37 @@
         <v>103</v>
       </c>
       <c r="D40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H40">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I40">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J40">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K40">
         <v>5</v>
       </c>
       <c r="L40">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M40">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N40">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O40">
         <v>6</v>
@@ -3411,37 +3411,37 @@
         <v>103</v>
       </c>
       <c r="D41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G41">
         <v>2</v>
       </c>
       <c r="H41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I41">
         <v>6</v>
       </c>
       <c r="J41">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K41">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L41">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M41">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N41">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O41">
         <v>6</v>
@@ -3479,37 +3479,37 @@
         <v>102</v>
       </c>
       <c r="D42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42">
         <v>2</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H42">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I42">
         <v>6</v>
       </c>
       <c r="J42">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K42">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L42">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M42">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N42">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O42">
         <v>6</v>
@@ -3550,34 +3550,34 @@
         <v>2</v>
       </c>
       <c r="E43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43">
         <v>2</v>
       </c>
       <c r="G43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H43">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I43">
         <v>5</v>
       </c>
       <c r="J43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L43">
         <v>5</v>
       </c>
       <c r="M43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N43">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O43">
         <v>6</v>
@@ -3615,34 +3615,34 @@
         <v>103</v>
       </c>
       <c r="D44">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F44">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G44">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H44">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I44">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K44">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L44">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N44">
         <v>3</v>
@@ -3683,37 +3683,37 @@
         <v>102</v>
       </c>
       <c r="D45">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E45">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G45">
         <v>2</v>
       </c>
       <c r="H45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I45">
         <v>4</v>
       </c>
       <c r="J45">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K45">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L45">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M45">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N45">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O45">
         <v>6</v>
@@ -3751,37 +3751,37 @@
         <v>103</v>
       </c>
       <c r="D46">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E46">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G46">
         <v>3</v>
       </c>
       <c r="H46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I46">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J46">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K46">
         <v>4</v>
       </c>
       <c r="L46">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M46">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="N46">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O46">
         <v>6</v>
@@ -3822,31 +3822,31 @@
         <v>2</v>
       </c>
       <c r="E47">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G47">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H47">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I47">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J47">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K47">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L47">
         <v>5</v>
       </c>
       <c r="M47">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N47">
         <v>5</v>
@@ -3887,37 +3887,37 @@
         <v>101</v>
       </c>
       <c r="D48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F48">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G48">
         <v>2</v>
       </c>
       <c r="H48">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N48">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O48">
         <v>6</v>
@@ -3955,19 +3955,19 @@
         <v>103</v>
       </c>
       <c r="D49">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I49">
         <v>4</v>
@@ -3976,16 +3976,16 @@
         <v>4</v>
       </c>
       <c r="K49">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L49">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M49">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N49">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O49">
         <v>6</v>
@@ -4023,37 +4023,37 @@
         <v>102</v>
       </c>
       <c r="D50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F50">
         <v>2</v>
       </c>
       <c r="G50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I50">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J50">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K50">
         <v>6</v>
       </c>
       <c r="L50">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M50">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N50">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O50">
         <v>6</v>
@@ -4091,37 +4091,37 @@
         <v>101</v>
       </c>
       <c r="D51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F51">
         <v>2</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I51">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J51">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K51">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L51">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M51">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N51">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O51">
         <v>6</v>
@@ -4165,16 +4165,16 @@
         <v>2</v>
       </c>
       <c r="F52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G52">
         <v>3</v>
       </c>
       <c r="H52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I52">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J52">
         <v>4</v>
@@ -4183,13 +4183,13 @@
         <v>5</v>
       </c>
       <c r="L52">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M52">
         <v>4</v>
       </c>
       <c r="N52">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O52">
         <v>6</v>
@@ -4227,16 +4227,16 @@
         <v>102</v>
       </c>
       <c r="D53">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F53">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G53">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H53">
         <v>2</v>
@@ -4248,16 +4248,16 @@
         <v>4</v>
       </c>
       <c r="K53">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L53">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M53">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N53">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O53">
         <v>6</v>
@@ -4295,37 +4295,37 @@
         <v>102</v>
       </c>
       <c r="D54">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G54">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H54">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I54">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J54">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K54">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L54">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M54">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N54">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O54">
         <v>6</v>
@@ -4363,37 +4363,37 @@
         <v>102</v>
       </c>
       <c r="D55">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E55">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F55">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G55">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H55">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I55">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J55">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K55">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L55">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M55">
         <v>6</v>
       </c>
       <c r="N55">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O55">
         <v>6</v>
@@ -4431,37 +4431,37 @@
         <v>102</v>
       </c>
       <c r="D56">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E56">
         <v>2</v>
       </c>
       <c r="F56">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G56">
         <v>3</v>
       </c>
       <c r="H56">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I56">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J56">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K56">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L56">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N56">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O56">
         <v>6</v>
@@ -4502,7 +4502,7 @@
         <v>2</v>
       </c>
       <c r="E57">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -4511,25 +4511,25 @@
         <v>1</v>
       </c>
       <c r="H57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I57">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J57">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K57">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L57">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M57">
         <v>6</v>
       </c>
       <c r="N57">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O57">
         <v>6</v>
@@ -4567,37 +4567,37 @@
         <v>103</v>
       </c>
       <c r="D58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F58">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G58">
         <v>3</v>
       </c>
       <c r="H58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L58">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O58">
         <v>6</v>
@@ -4635,10 +4635,10 @@
         <v>102</v>
       </c>
       <c r="D59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E59">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F59">
         <v>3</v>
@@ -4650,19 +4650,19 @@
         <v>3</v>
       </c>
       <c r="I59">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J59">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K59">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L59">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M59">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N59">
         <v>5</v>
@@ -4703,37 +4703,37 @@
         <v>101</v>
       </c>
       <c r="D60">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E60">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F60">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G60">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H60">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I60">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J60">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K60">
         <v>3</v>
       </c>
       <c r="L60">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M60">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N60">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O60">
         <v>6</v>
@@ -4771,37 +4771,37 @@
         <v>103</v>
       </c>
       <c r="D61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E61">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F61">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G61">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H61">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I61">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J61">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K61">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L61">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M61">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N61">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O61">
         <v>6</v>
@@ -4842,34 +4842,34 @@
         <v>2</v>
       </c>
       <c r="E62">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H62">
         <v>2</v>
       </c>
       <c r="I62">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J62">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K62">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L62">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M62">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N62">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O62">
         <v>6</v>
@@ -4907,13 +4907,13 @@
         <v>101</v>
       </c>
       <c r="D63">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E63">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G63">
         <v>4</v>
@@ -4922,22 +4922,22 @@
         <v>3</v>
       </c>
       <c r="I63">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J63">
         <v>4</v>
       </c>
       <c r="K63">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L63">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M63">
         <v>4</v>
       </c>
       <c r="N63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O63">
         <v>6</v>
@@ -4975,34 +4975,34 @@
         <v>101</v>
       </c>
       <c r="D64">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E64">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F64">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G64">
         <v>2</v>
       </c>
       <c r="H64">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I64">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J64">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K64">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L64">
         <v>5</v>
       </c>
       <c r="M64">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N64">
         <v>5</v>
@@ -5040,37 +5040,37 @@
         <v>101</v>
       </c>
       <c r="D65">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E65">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F65">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H65">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I65">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J65">
         <v>5</v>
       </c>
       <c r="K65">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L65">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M65">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N65">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O65">
         <v>6</v>
@@ -5108,37 +5108,37 @@
         <v>101</v>
       </c>
       <c r="D66">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E66">
         <v>4</v>
       </c>
       <c r="F66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H66">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I66">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J66">
         <v>4</v>
       </c>
       <c r="K66">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M66">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N66">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O66">
         <v>6</v>
@@ -5179,22 +5179,22 @@
         <v>1</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H67">
         <v>2</v>
       </c>
       <c r="I67">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J67">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K67">
         <v>5</v>
@@ -5203,10 +5203,10 @@
         <v>6</v>
       </c>
       <c r="M67">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N67">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O67">
         <v>6</v>
@@ -5244,37 +5244,37 @@
         <v>102</v>
       </c>
       <c r="D68">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E68">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F68">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G68">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H68">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K68">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M68">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O68">
         <v>6</v>
@@ -5312,34 +5312,34 @@
         <v>101</v>
       </c>
       <c r="D69">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H69">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J69">
         <v>4</v>
       </c>
       <c r="K69">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N69">
         <v>4</v>
@@ -5380,34 +5380,34 @@
         <v>102</v>
       </c>
       <c r="D70">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F70">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G70">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H70">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I70">
         <v>5</v>
       </c>
       <c r="J70">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K70">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L70">
         <v>5</v>
       </c>
       <c r="M70">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N70">
         <v>5</v>
@@ -5448,37 +5448,37 @@
         <v>103</v>
       </c>
       <c r="D71">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E71">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F71">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G71">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H71">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I71">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J71">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K71">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L71">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M71">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N71">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O71">
         <v>6</v>
@@ -5516,34 +5516,34 @@
         <v>101</v>
       </c>
       <c r="D72">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E72">
         <v>3</v>
       </c>
       <c r="F72">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G72">
         <v>2</v>
       </c>
       <c r="H72">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I72">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J72">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K72">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L72">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M72">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N72">
         <v>4</v>
@@ -5584,37 +5584,37 @@
         <v>102</v>
       </c>
       <c r="D73">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G73">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H73">
         <v>2</v>
       </c>
       <c r="I73">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J73">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K73">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L73">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M73">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N73">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O73">
         <v>6</v>
@@ -5652,37 +5652,37 @@
         <v>101</v>
       </c>
       <c r="D74">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F74">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I74">
         <v>4</v>
       </c>
       <c r="J74">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K74">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L74">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M74">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N74">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O74">
         <v>6</v>
@@ -5720,37 +5720,37 @@
         <v>101</v>
       </c>
       <c r="D75">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F75">
         <v>2</v>
       </c>
       <c r="G75">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H75">
         <v>2</v>
       </c>
       <c r="I75">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J75">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K75">
         <v>5</v>
       </c>
       <c r="L75">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M75">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N75">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O75">
         <v>6</v>
@@ -5788,13 +5788,13 @@
         <v>101</v>
       </c>
       <c r="D76">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E76">
         <v>3</v>
       </c>
       <c r="F76">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G76">
         <v>2</v>
@@ -5803,22 +5803,22 @@
         <v>2</v>
       </c>
       <c r="I76">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J76">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K76">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L76">
         <v>5</v>
       </c>
       <c r="M76">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N76">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O76">
         <v>6</v>
@@ -5856,7 +5856,7 @@
         <v>103</v>
       </c>
       <c r="D77">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -5865,25 +5865,25 @@
         <v>3</v>
       </c>
       <c r="G77">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H77">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I77">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J77">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K77">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L77">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M77">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N77">
         <v>5</v>
@@ -5924,37 +5924,37 @@
         <v>103</v>
       </c>
       <c r="D78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E78">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G78">
         <v>2</v>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I78">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J78">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K78">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L78">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M78">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N78">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O78">
         <v>6</v>
@@ -5992,37 +5992,37 @@
         <v>101</v>
       </c>
       <c r="D79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E79">
         <v>3</v>
       </c>
       <c r="F79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G79">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I79">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J79">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K79">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L79">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M79">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N79">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O79">
         <v>6</v>
@@ -6063,34 +6063,34 @@
         <v>4</v>
       </c>
       <c r="E80">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F80">
         <v>3</v>
       </c>
       <c r="G80">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H80">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I80">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J80">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K80">
         <v>4</v>
       </c>
       <c r="L80">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M80">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N80">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O80">
         <v>6</v>

</xml_diff>

<commit_message>
data v7.0: leader-rated OCBS/CWBS realistic ICC (~0.27/0.22)
</commit_message>
<xml_diff>
--- a/data/T3_leader_cleaned.xlsx
+++ b/data/T3_leader_cleaned.xlsx
@@ -765,37 +765,37 @@
         <v>101</v>
       </c>
       <c r="D2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J2">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M2">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O2">
         <v>6</v>
@@ -833,37 +833,37 @@
         <v>101</v>
       </c>
       <c r="D3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>2</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I3">
         <v>6</v>
       </c>
       <c r="J3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L3">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M3">
         <v>6</v>
       </c>
       <c r="N3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O3">
         <v>6</v>
@@ -904,34 +904,34 @@
         <v>4</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O4">
         <v>6</v>
@@ -969,37 +969,37 @@
         <v>102</v>
       </c>
       <c r="D5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L5">
         <v>5</v>
       </c>
       <c r="M5">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O5">
         <v>6</v>
@@ -1037,37 +1037,37 @@
         <v>102</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O6">
         <v>6</v>
@@ -1105,37 +1105,37 @@
         <v>103</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E7">
         <v>2</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="H7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I7">
         <v>4</v>
       </c>
       <c r="J7">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O7">
         <v>6</v>
@@ -1173,37 +1173,37 @@
         <v>103</v>
       </c>
       <c r="D8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H8">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O8">
         <v>6</v>
@@ -1241,19 +1241,19 @@
         <v>101</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I9">
         <v>4</v>
@@ -1265,13 +1265,13 @@
         <v>4</v>
       </c>
       <c r="L9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O9">
         <v>6</v>
@@ -1309,10 +1309,10 @@
         <v>101</v>
       </c>
       <c r="D10">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F10">
         <v>3</v>
@@ -1324,16 +1324,16 @@
         <v>3</v>
       </c>
       <c r="I10">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K10">
         <v>4</v>
       </c>
       <c r="L10">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M10">
         <v>4</v>
@@ -1377,31 +1377,31 @@
         <v>102</v>
       </c>
       <c r="D11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E11">
         <v>4</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G11">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H11">
         <v>4</v>
       </c>
       <c r="I11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K11">
         <v>5</v>
       </c>
       <c r="L11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M11">
         <v>5</v>
@@ -1445,10 +1445,10 @@
         <v>102</v>
       </c>
       <c r="D12">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F12">
         <v>3</v>
@@ -1457,19 +1457,19 @@
         <v>2</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I12">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M12">
         <v>5</v>
@@ -1516,16 +1516,16 @@
         <v>3</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13">
         <v>3</v>
       </c>
       <c r="G13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I13">
         <v>5</v>
@@ -1534,16 +1534,16 @@
         <v>4</v>
       </c>
       <c r="K13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L13">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M13">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N13">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O13">
         <v>6</v>
@@ -1581,37 +1581,37 @@
         <v>102</v>
       </c>
       <c r="D14">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E14">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F14">
         <v>2</v>
       </c>
       <c r="G14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H14">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="I14">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K14">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M14">
         <v>3</v>
       </c>
       <c r="N14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O14">
         <v>6</v>
@@ -1649,31 +1649,31 @@
         <v>102</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E15">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F15">
         <v>3</v>
       </c>
       <c r="G15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M15">
         <v>4</v>
@@ -1714,28 +1714,28 @@
         <v>102</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J16">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K16">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L16">
         <v>4</v>
@@ -1785,34 +1785,34 @@
         <v>3</v>
       </c>
       <c r="E17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I17">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K17">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L17">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M17">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N17">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O17">
         <v>6</v>
@@ -1850,37 +1850,37 @@
         <v>101</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I18">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N18">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O18">
         <v>6</v>
@@ -1918,22 +1918,22 @@
         <v>103</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G19">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H19">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I19">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J19">
         <v>5</v>
@@ -1942,13 +1942,13 @@
         <v>6</v>
       </c>
       <c r="L19">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M19">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N19">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O19">
         <v>6</v>
@@ -1986,37 +1986,37 @@
         <v>101</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G20">
         <v>2</v>
       </c>
       <c r="H20">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K20">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L20">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M20">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N20">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O20">
         <v>6</v>
@@ -2054,34 +2054,34 @@
         <v>103</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I21">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L21">
         <v>4</v>
       </c>
       <c r="M21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N21">
         <v>5</v>
@@ -2122,34 +2122,34 @@
         <v>102</v>
       </c>
       <c r="D22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22">
         <v>2</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I22">
         <v>5</v>
       </c>
       <c r="J22">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K22">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="L22">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N22">
         <v>6</v>
@@ -2190,13 +2190,13 @@
         <v>103</v>
       </c>
       <c r="D23">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E23">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F23">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G23">
         <v>2</v>
@@ -2205,13 +2205,13 @@
         <v>3</v>
       </c>
       <c r="I23">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J23">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K23">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L23">
         <v>5</v>
@@ -2261,34 +2261,34 @@
         <v>3</v>
       </c>
       <c r="E24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I24">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J24">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L24">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N24">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O24">
         <v>6</v>
@@ -2323,37 +2323,37 @@
         <v>101</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G25">
         <v>2</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J25">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K25">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N25">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O25">
         <v>6</v>
@@ -2391,19 +2391,19 @@
         <v>103</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I26">
         <v>4</v>
@@ -2412,16 +2412,16 @@
         <v>5</v>
       </c>
       <c r="K26">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L26">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N26">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O26">
         <v>6</v>
@@ -2459,31 +2459,31 @@
         <v>103</v>
       </c>
       <c r="D27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G27">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I27">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J27">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K27">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L27">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M27">
         <v>5</v>
@@ -2530,16 +2530,16 @@
         <v>2</v>
       </c>
       <c r="E28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I28">
         <v>5</v>
@@ -2548,13 +2548,13 @@
         <v>5</v>
       </c>
       <c r="K28">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N28">
         <v>5</v>
@@ -2595,37 +2595,37 @@
         <v>102</v>
       </c>
       <c r="D29">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E29">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G29">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I29">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L29">
         <v>4</v>
       </c>
       <c r="M29">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N29">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O29">
         <v>6</v>
@@ -2663,22 +2663,22 @@
         <v>101</v>
       </c>
       <c r="D30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E30">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H30">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I30">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J30">
         <v>4</v>
@@ -2687,13 +2687,13 @@
         <v>4</v>
       </c>
       <c r="L30">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M30">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N30">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O30">
         <v>6</v>
@@ -2731,37 +2731,37 @@
         <v>103</v>
       </c>
       <c r="D31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F31">
         <v>3</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J31">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K31">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O31">
         <v>6</v>
@@ -2799,37 +2799,37 @@
         <v>101</v>
       </c>
       <c r="D32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32">
         <v>2</v>
       </c>
       <c r="G32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H32">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L32">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O32">
         <v>6</v>
@@ -2870,34 +2870,34 @@
         <v>2</v>
       </c>
       <c r="E33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H33">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I33">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J33">
         <v>5</v>
       </c>
       <c r="K33">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M33">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N33">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O33">
         <v>6</v>
@@ -2935,37 +2935,37 @@
         <v>102</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E34">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I34">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J34">
         <v>5</v>
       </c>
       <c r="K34">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L34">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M34">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N34">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O34">
         <v>6</v>
@@ -3003,37 +3003,37 @@
         <v>103</v>
       </c>
       <c r="D35">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G35">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H35">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J35">
         <v>4</v>
       </c>
       <c r="K35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L35">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N35">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O35">
         <v>6</v>
@@ -3071,37 +3071,37 @@
         <v>102</v>
       </c>
       <c r="D36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F36">
         <v>2</v>
       </c>
       <c r="G36">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L36">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N36">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O36">
         <v>6</v>
@@ -3139,37 +3139,37 @@
         <v>102</v>
       </c>
       <c r="D37">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F37">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G37">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H37">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I37">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J37">
         <v>5</v>
       </c>
       <c r="K37">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L37">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M37">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N37">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O37">
         <v>6</v>
@@ -3207,37 +3207,37 @@
         <v>103</v>
       </c>
       <c r="D38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E38">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G38">
         <v>3</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I38">
         <v>3</v>
       </c>
       <c r="J38">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K38">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L38">
         <v>3</v>
       </c>
       <c r="M38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N38">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O38">
         <v>6</v>
@@ -3275,10 +3275,10 @@
         <v>101</v>
       </c>
       <c r="D39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E39">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F39">
         <v>3</v>
@@ -3290,22 +3290,22 @@
         <v>3</v>
       </c>
       <c r="I39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K39">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L39">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M39">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N39">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O39">
         <v>6</v>
@@ -3343,37 +3343,37 @@
         <v>103</v>
       </c>
       <c r="D40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E40">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H40">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I40">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J40">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K40">
         <v>5</v>
       </c>
       <c r="L40">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M40">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N40">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O40">
         <v>6</v>
@@ -3411,37 +3411,37 @@
         <v>103</v>
       </c>
       <c r="D41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G41">
         <v>2</v>
       </c>
       <c r="H41">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I41">
         <v>6</v>
       </c>
       <c r="J41">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K41">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L41">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M41">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N41">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O41">
         <v>6</v>
@@ -3479,37 +3479,37 @@
         <v>102</v>
       </c>
       <c r="D42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F42">
         <v>2</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H42">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I42">
         <v>6</v>
       </c>
       <c r="J42">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K42">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L42">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M42">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N42">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O42">
         <v>6</v>
@@ -3550,34 +3550,34 @@
         <v>2</v>
       </c>
       <c r="E43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43">
         <v>2</v>
       </c>
       <c r="G43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H43">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I43">
         <v>5</v>
       </c>
       <c r="J43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L43">
         <v>5</v>
       </c>
       <c r="M43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N43">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O43">
         <v>6</v>
@@ -3615,34 +3615,34 @@
         <v>103</v>
       </c>
       <c r="D44">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E44">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F44">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G44">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H44">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I44">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K44">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L44">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="M44">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N44">
         <v>3</v>
@@ -3683,37 +3683,37 @@
         <v>102</v>
       </c>
       <c r="D45">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E45">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G45">
         <v>2</v>
       </c>
       <c r="H45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I45">
         <v>4</v>
       </c>
       <c r="J45">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K45">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L45">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M45">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N45">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O45">
         <v>6</v>
@@ -3751,37 +3751,37 @@
         <v>103</v>
       </c>
       <c r="D46">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E46">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G46">
         <v>3</v>
       </c>
       <c r="H46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I46">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J46">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K46">
         <v>4</v>
       </c>
       <c r="L46">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M46">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="N46">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O46">
         <v>6</v>
@@ -3822,31 +3822,31 @@
         <v>2</v>
       </c>
       <c r="E47">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G47">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H47">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I47">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J47">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K47">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L47">
         <v>5</v>
       </c>
       <c r="M47">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N47">
         <v>5</v>
@@ -3887,37 +3887,37 @@
         <v>101</v>
       </c>
       <c r="D48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F48">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G48">
         <v>2</v>
       </c>
       <c r="H48">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M48">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N48">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O48">
         <v>6</v>
@@ -3955,19 +3955,19 @@
         <v>103</v>
       </c>
       <c r="D49">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H49">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I49">
         <v>4</v>
@@ -3976,16 +3976,16 @@
         <v>4</v>
       </c>
       <c r="K49">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L49">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M49">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N49">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O49">
         <v>6</v>
@@ -4023,37 +4023,37 @@
         <v>102</v>
       </c>
       <c r="D50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F50">
         <v>2</v>
       </c>
       <c r="G50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I50">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J50">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K50">
         <v>6</v>
       </c>
       <c r="L50">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M50">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N50">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="O50">
         <v>6</v>
@@ -4091,37 +4091,37 @@
         <v>101</v>
       </c>
       <c r="D51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F51">
         <v>2</v>
       </c>
       <c r="G51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I51">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J51">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K51">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L51">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M51">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N51">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O51">
         <v>6</v>
@@ -4165,16 +4165,16 @@
         <v>2</v>
       </c>
       <c r="F52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G52">
         <v>3</v>
       </c>
       <c r="H52">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I52">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J52">
         <v>4</v>
@@ -4183,13 +4183,13 @@
         <v>5</v>
       </c>
       <c r="L52">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M52">
         <v>4</v>
       </c>
       <c r="N52">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O52">
         <v>6</v>
@@ -4227,16 +4227,16 @@
         <v>102</v>
       </c>
       <c r="D53">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E53">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F53">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G53">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H53">
         <v>2</v>
@@ -4248,16 +4248,16 @@
         <v>4</v>
       </c>
       <c r="K53">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L53">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M53">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N53">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O53">
         <v>6</v>
@@ -4295,37 +4295,37 @@
         <v>102</v>
       </c>
       <c r="D54">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G54">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H54">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I54">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J54">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K54">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L54">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M54">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N54">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O54">
         <v>6</v>
@@ -4363,37 +4363,37 @@
         <v>102</v>
       </c>
       <c r="D55">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E55">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F55">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G55">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H55">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I55">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J55">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K55">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L55">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M55">
         <v>6</v>
       </c>
       <c r="N55">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O55">
         <v>6</v>
@@ -4431,37 +4431,37 @@
         <v>102</v>
       </c>
       <c r="D56">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E56">
         <v>2</v>
       </c>
       <c r="F56">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G56">
         <v>3</v>
       </c>
       <c r="H56">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I56">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J56">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K56">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L56">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N56">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O56">
         <v>6</v>
@@ -4502,7 +4502,7 @@
         <v>2</v>
       </c>
       <c r="E57">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F57">
         <v>1</v>
@@ -4511,25 +4511,25 @@
         <v>1</v>
       </c>
       <c r="H57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I57">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J57">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K57">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L57">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M57">
         <v>6</v>
       </c>
       <c r="N57">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O57">
         <v>6</v>
@@ -4567,37 +4567,37 @@
         <v>103</v>
       </c>
       <c r="D58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F58">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G58">
         <v>3</v>
       </c>
       <c r="H58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L58">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O58">
         <v>6</v>
@@ -4635,10 +4635,10 @@
         <v>102</v>
       </c>
       <c r="D59">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E59">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F59">
         <v>3</v>
@@ -4650,19 +4650,19 @@
         <v>3</v>
       </c>
       <c r="I59">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J59">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K59">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L59">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M59">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N59">
         <v>5</v>
@@ -4703,37 +4703,37 @@
         <v>101</v>
       </c>
       <c r="D60">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E60">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F60">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G60">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H60">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I60">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J60">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K60">
         <v>3</v>
       </c>
       <c r="L60">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M60">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N60">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="O60">
         <v>6</v>
@@ -4771,37 +4771,37 @@
         <v>103</v>
       </c>
       <c r="D61">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E61">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F61">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G61">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H61">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I61">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J61">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K61">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L61">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M61">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N61">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O61">
         <v>6</v>
@@ -4842,34 +4842,34 @@
         <v>2</v>
       </c>
       <c r="E62">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F62">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H62">
         <v>2</v>
       </c>
       <c r="I62">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J62">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K62">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L62">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M62">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N62">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O62">
         <v>6</v>
@@ -4907,13 +4907,13 @@
         <v>101</v>
       </c>
       <c r="D63">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E63">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F63">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G63">
         <v>4</v>
@@ -4922,22 +4922,22 @@
         <v>3</v>
       </c>
       <c r="I63">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J63">
         <v>4</v>
       </c>
       <c r="K63">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L63">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M63">
         <v>4</v>
       </c>
       <c r="N63">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O63">
         <v>6</v>
@@ -4975,34 +4975,34 @@
         <v>101</v>
       </c>
       <c r="D64">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E64">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F64">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G64">
         <v>2</v>
       </c>
       <c r="H64">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I64">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J64">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K64">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L64">
         <v>5</v>
       </c>
       <c r="M64">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N64">
         <v>5</v>
@@ -5040,37 +5040,37 @@
         <v>101</v>
       </c>
       <c r="D65">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E65">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F65">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H65">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I65">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J65">
         <v>5</v>
       </c>
       <c r="K65">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L65">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="M65">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N65">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O65">
         <v>6</v>
@@ -5108,37 +5108,37 @@
         <v>101</v>
       </c>
       <c r="D66">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E66">
         <v>4</v>
       </c>
       <c r="F66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H66">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I66">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J66">
         <v>4</v>
       </c>
       <c r="K66">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M66">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N66">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O66">
         <v>6</v>
@@ -5179,22 +5179,22 @@
         <v>1</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H67">
         <v>2</v>
       </c>
       <c r="I67">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J67">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K67">
         <v>5</v>
@@ -5203,10 +5203,10 @@
         <v>6</v>
       </c>
       <c r="M67">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N67">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O67">
         <v>6</v>
@@ -5244,37 +5244,37 @@
         <v>102</v>
       </c>
       <c r="D68">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E68">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F68">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G68">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H68">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K68">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M68">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N68">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O68">
         <v>6</v>
@@ -5312,34 +5312,34 @@
         <v>101</v>
       </c>
       <c r="D69">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H69">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J69">
         <v>4</v>
       </c>
       <c r="K69">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N69">
         <v>4</v>
@@ -5380,34 +5380,34 @@
         <v>102</v>
       </c>
       <c r="D70">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E70">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F70">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G70">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H70">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I70">
         <v>5</v>
       </c>
       <c r="J70">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K70">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L70">
         <v>5</v>
       </c>
       <c r="M70">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N70">
         <v>5</v>
@@ -5448,37 +5448,37 @@
         <v>103</v>
       </c>
       <c r="D71">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E71">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F71">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G71">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H71">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I71">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J71">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K71">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L71">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M71">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N71">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O71">
         <v>6</v>
@@ -5516,34 +5516,34 @@
         <v>101</v>
       </c>
       <c r="D72">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E72">
         <v>3</v>
       </c>
       <c r="F72">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G72">
         <v>2</v>
       </c>
       <c r="H72">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I72">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J72">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K72">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L72">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M72">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N72">
         <v>4</v>
@@ -5584,37 +5584,37 @@
         <v>102</v>
       </c>
       <c r="D73">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G73">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H73">
         <v>2</v>
       </c>
       <c r="I73">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J73">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K73">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L73">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M73">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N73">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O73">
         <v>6</v>
@@ -5652,37 +5652,37 @@
         <v>101</v>
       </c>
       <c r="D74">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F74">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H74">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I74">
         <v>4</v>
       </c>
       <c r="J74">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K74">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L74">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M74">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N74">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O74">
         <v>6</v>
@@ -5720,37 +5720,37 @@
         <v>101</v>
       </c>
       <c r="D75">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F75">
         <v>2</v>
       </c>
       <c r="G75">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H75">
         <v>2</v>
       </c>
       <c r="I75">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J75">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K75">
         <v>5</v>
       </c>
       <c r="L75">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M75">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N75">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O75">
         <v>6</v>
@@ -5788,13 +5788,13 @@
         <v>101</v>
       </c>
       <c r="D76">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E76">
         <v>3</v>
       </c>
       <c r="F76">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G76">
         <v>2</v>
@@ -5803,22 +5803,22 @@
         <v>2</v>
       </c>
       <c r="I76">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J76">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K76">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L76">
         <v>5</v>
       </c>
       <c r="M76">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N76">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="O76">
         <v>6</v>
@@ -5856,7 +5856,7 @@
         <v>103</v>
       </c>
       <c r="D77">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E77">
         <v>2</v>
@@ -5865,25 +5865,25 @@
         <v>3</v>
       </c>
       <c r="G77">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H77">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I77">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J77">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K77">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L77">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M77">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N77">
         <v>5</v>
@@ -5924,37 +5924,37 @@
         <v>103</v>
       </c>
       <c r="D78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E78">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G78">
         <v>2</v>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I78">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J78">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K78">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="L78">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M78">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N78">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O78">
         <v>6</v>
@@ -5992,37 +5992,37 @@
         <v>101</v>
       </c>
       <c r="D79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E79">
         <v>3</v>
       </c>
       <c r="F79">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G79">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H79">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I79">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J79">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="K79">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L79">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M79">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="N79">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O79">
         <v>6</v>
@@ -6063,34 +6063,34 @@
         <v>4</v>
       </c>
       <c r="E80">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F80">
         <v>3</v>
       </c>
       <c r="G80">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H80">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I80">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J80">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K80">
         <v>4</v>
       </c>
       <c r="L80">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M80">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N80">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O80">
         <v>6</v>

</xml_diff>

<commit_message>
round-4: rebuild N=361->340 (teams 10/35/34) + mirror-break correlations; derive Path/IE/slope tables from genuine lme4 raw output (fixes A29 inconsistent/identical coefficients); ship raw R code+output; validators 219/219 + audit 10/10
</commit_message>
<xml_diff>
--- a/data/T3_leader_cleaned.xlsx
+++ b/data/T3_leader_cleaned.xlsx
@@ -765,22 +765,22 @@
         <v>101</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>3</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J2">
         <v>4</v>
@@ -789,13 +789,13 @@
         <v>3</v>
       </c>
       <c r="L2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M2">
         <v>3</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>6</v>
@@ -836,34 +836,34 @@
         <v>2</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3">
         <v>2</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O3">
         <v>6</v>
@@ -904,7 +904,7 @@
         <v>4</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4">
         <v>4</v>
@@ -916,22 +916,22 @@
         <v>4</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K4">
         <v>5</v>
       </c>
       <c r="L4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O4">
         <v>6</v>
@@ -972,25 +972,25 @@
         <v>2</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I5">
         <v>5</v>
       </c>
       <c r="J5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -1037,13 +1037,13 @@
         <v>102</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G6">
         <v>3</v>
@@ -1055,19 +1055,19 @@
         <v>4</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M6">
         <v>4</v>
       </c>
       <c r="N6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O6">
         <v>6</v>
@@ -1108,34 +1108,34 @@
         <v>3</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O7">
         <v>6</v>
@@ -1173,10 +1173,10 @@
         <v>103</v>
       </c>
       <c r="D8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8">
         <v>4</v>
@@ -1185,25 +1185,25 @@
         <v>4</v>
       </c>
       <c r="H8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O8">
         <v>6</v>
@@ -1241,34 +1241,34 @@
         <v>101</v>
       </c>
       <c r="D9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M9">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N9">
         <v>4</v>
@@ -1309,37 +1309,37 @@
         <v>101</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10">
         <v>2</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O10">
         <v>6</v>
@@ -1386,7 +1386,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H11">
         <v>4</v>
@@ -1398,13 +1398,13 @@
         <v>5</v>
       </c>
       <c r="K11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L11">
         <v>5</v>
       </c>
       <c r="M11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N11">
         <v>5</v>
@@ -1451,31 +1451,31 @@
         <v>3</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H12">
         <v>3</v>
       </c>
       <c r="I12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J12">
         <v>5</v>
       </c>
       <c r="K12">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O12">
         <v>6</v>
@@ -1513,37 +1513,37 @@
         <v>103</v>
       </c>
       <c r="D13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G13">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13">
         <v>4</v>
       </c>
       <c r="K13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M13">
         <v>4</v>
       </c>
       <c r="N13">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O13">
         <v>6</v>
@@ -1581,37 +1581,37 @@
         <v>102</v>
       </c>
       <c r="D14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K14">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O14">
         <v>6</v>
@@ -1658,10 +1658,10 @@
         <v>3</v>
       </c>
       <c r="G15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I15">
         <v>4</v>
@@ -1670,7 +1670,7 @@
         <v>4</v>
       </c>
       <c r="K15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L15">
         <v>4</v>
@@ -1714,37 +1714,37 @@
         <v>102</v>
       </c>
       <c r="D16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O16">
         <v>6</v>
@@ -1785,34 +1785,34 @@
         <v>3</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17">
         <v>3</v>
       </c>
       <c r="G17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I17">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J17">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K17">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M17">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N17">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O17">
         <v>6</v>
@@ -1850,19 +1850,19 @@
         <v>101</v>
       </c>
       <c r="D18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I18">
         <v>5</v>
@@ -1874,13 +1874,13 @@
         <v>5</v>
       </c>
       <c r="L18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O18">
         <v>6</v>
@@ -1918,28 +1918,28 @@
         <v>103</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G19">
         <v>3</v>
       </c>
       <c r="H19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I19">
         <v>6</v>
       </c>
       <c r="J19">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L19">
         <v>5</v>
@@ -1948,7 +1948,7 @@
         <v>5</v>
       </c>
       <c r="N19">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O19">
         <v>6</v>
@@ -1998,25 +1998,25 @@
         <v>2</v>
       </c>
       <c r="H20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J20">
         <v>5</v>
       </c>
       <c r="K20">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L20">
         <v>5</v>
       </c>
       <c r="M20">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N20">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O20">
         <v>6</v>
@@ -2054,7 +2054,7 @@
         <v>103</v>
       </c>
       <c r="D21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E21">
         <v>2</v>
@@ -2069,22 +2069,22 @@
         <v>3</v>
       </c>
       <c r="I21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J21">
         <v>5</v>
       </c>
       <c r="K21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L21">
         <v>4</v>
       </c>
       <c r="M21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O21">
         <v>6</v>
@@ -2122,7 +2122,7 @@
         <v>102</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22">
         <v>2</v>
@@ -2134,25 +2134,25 @@
         <v>2</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I22">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J22">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K22">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L22">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M22">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N22">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O22">
         <v>6</v>
@@ -2193,7 +2193,7 @@
         <v>2</v>
       </c>
       <c r="E23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23">
         <v>2</v>
@@ -2202,7 +2202,7 @@
         <v>2</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I23">
         <v>6</v>
@@ -2214,7 +2214,7 @@
         <v>5</v>
       </c>
       <c r="L23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M23">
         <v>6</v>
@@ -2261,13 +2261,13 @@
         <v>3</v>
       </c>
       <c r="E24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F24">
         <v>3</v>
       </c>
       <c r="G24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H24">
         <v>3</v>
@@ -2276,13 +2276,13 @@
         <v>5</v>
       </c>
       <c r="J24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M24">
         <v>5</v>
@@ -2329,31 +2329,31 @@
         <v>2</v>
       </c>
       <c r="F25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G25">
         <v>2</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L25">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N25">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O25">
         <v>6</v>
@@ -2391,37 +2391,37 @@
         <v>103</v>
       </c>
       <c r="D26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26">
         <v>2</v>
       </c>
       <c r="G26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L26">
         <v>4</v>
       </c>
       <c r="M26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O26">
         <v>6</v>
@@ -2474,16 +2474,16 @@
         <v>2</v>
       </c>
       <c r="I27">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K27">
         <v>5</v>
       </c>
       <c r="L27">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M27">
         <v>5</v>
@@ -2527,13 +2527,13 @@
         <v>101</v>
       </c>
       <c r="D28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G28">
         <v>3</v>
@@ -2542,22 +2542,22 @@
         <v>3</v>
       </c>
       <c r="I28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M28">
         <v>5</v>
       </c>
       <c r="N28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O28">
         <v>6</v>
@@ -2604,25 +2604,25 @@
         <v>2</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J29">
         <v>4</v>
       </c>
       <c r="K29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L29">
         <v>4</v>
       </c>
       <c r="M29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N29">
         <v>4</v>
@@ -2669,7 +2669,7 @@
         <v>2</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G30">
         <v>2</v>
@@ -2678,22 +2678,22 @@
         <v>2</v>
       </c>
       <c r="I30">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J30">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K30">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N30">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O30">
         <v>6</v>
@@ -2731,16 +2731,16 @@
         <v>103</v>
       </c>
       <c r="D31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31">
         <v>3</v>
       </c>
       <c r="F31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H31">
         <v>2</v>
@@ -2749,19 +2749,19 @@
         <v>4</v>
       </c>
       <c r="J31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K31">
         <v>4</v>
       </c>
       <c r="L31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O31">
         <v>6</v>
@@ -2799,37 +2799,37 @@
         <v>101</v>
       </c>
       <c r="D32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M32">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O32">
         <v>6</v>
@@ -2867,37 +2867,37 @@
         <v>103</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I33">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J33">
         <v>5</v>
       </c>
       <c r="K33">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L33">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M33">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N33">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O33">
         <v>6</v>
@@ -2938,7 +2938,7 @@
         <v>2</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F34">
         <v>2</v>
@@ -2950,16 +2950,16 @@
         <v>2</v>
       </c>
       <c r="I34">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K34">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M34">
         <v>5</v>
@@ -3006,7 +3006,7 @@
         <v>4</v>
       </c>
       <c r="E35">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -3015,7 +3015,7 @@
         <v>4</v>
       </c>
       <c r="H35">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I35">
         <v>4</v>
@@ -3071,31 +3071,31 @@
         <v>102</v>
       </c>
       <c r="D36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K36">
         <v>5</v>
       </c>
       <c r="L36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M36">
         <v>5</v>
@@ -3139,22 +3139,22 @@
         <v>102</v>
       </c>
       <c r="D37">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E37">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H37">
         <v>3</v>
       </c>
       <c r="I37">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J37">
         <v>5</v>
@@ -3163,10 +3163,10 @@
         <v>5</v>
       </c>
       <c r="L37">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M37">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N37">
         <v>4</v>
@@ -3207,28 +3207,28 @@
         <v>103</v>
       </c>
       <c r="D38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G38">
         <v>3</v>
       </c>
       <c r="H38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I38">
         <v>3</v>
       </c>
       <c r="J38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L38">
         <v>3</v>
@@ -3237,7 +3237,7 @@
         <v>3</v>
       </c>
       <c r="N38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O38">
         <v>6</v>
@@ -3278,19 +3278,19 @@
         <v>2</v>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F39">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G39">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H39">
         <v>3</v>
       </c>
       <c r="I39">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J39">
         <v>5</v>
@@ -3299,13 +3299,13 @@
         <v>6</v>
       </c>
       <c r="L39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M39">
         <v>5</v>
       </c>
       <c r="N39">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O39">
         <v>6</v>
@@ -3343,22 +3343,22 @@
         <v>103</v>
       </c>
       <c r="D40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I40">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J40">
         <v>5</v>
@@ -3370,10 +3370,10 @@
         <v>5</v>
       </c>
       <c r="M40">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N40">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O40">
         <v>6</v>
@@ -3411,13 +3411,13 @@
         <v>103</v>
       </c>
       <c r="D41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41">
         <v>2</v>
       </c>
       <c r="F41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G41">
         <v>2</v>
@@ -3426,22 +3426,22 @@
         <v>2</v>
       </c>
       <c r="I41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M41">
         <v>6</v>
       </c>
       <c r="N41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O41">
         <v>6</v>
@@ -3479,25 +3479,25 @@
         <v>102</v>
       </c>
       <c r="D42">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G42">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H42">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I42">
         <v>6</v>
       </c>
       <c r="J42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K42">
         <v>5</v>
@@ -3506,7 +3506,7 @@
         <v>5</v>
       </c>
       <c r="M42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N42">
         <v>5</v>
@@ -3559,19 +3559,19 @@
         <v>2</v>
       </c>
       <c r="H43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M43">
         <v>6</v>
@@ -3615,37 +3615,37 @@
         <v>103</v>
       </c>
       <c r="D44">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E44">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F44">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G44">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H44">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O44">
         <v>6</v>
@@ -3692,7 +3692,7 @@
         <v>2</v>
       </c>
       <c r="G45">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H45">
         <v>2</v>
@@ -3701,7 +3701,7 @@
         <v>4</v>
       </c>
       <c r="J45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K45">
         <v>4</v>
@@ -3710,10 +3710,10 @@
         <v>4</v>
       </c>
       <c r="M45">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N45">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O45">
         <v>6</v>
@@ -3754,7 +3754,7 @@
         <v>3</v>
       </c>
       <c r="E46">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F46">
         <v>3</v>
@@ -3763,25 +3763,25 @@
         <v>3</v>
       </c>
       <c r="H46">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I46">
         <v>4</v>
       </c>
       <c r="J46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L46">
         <v>4</v>
       </c>
       <c r="M46">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O46">
         <v>6</v>
@@ -3819,10 +3819,10 @@
         <v>102</v>
       </c>
       <c r="D47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E47">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F47">
         <v>3</v>
@@ -3831,25 +3831,25 @@
         <v>2</v>
       </c>
       <c r="H47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K47">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L47">
         <v>5</v>
       </c>
       <c r="M47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O47">
         <v>6</v>
@@ -3887,19 +3887,19 @@
         <v>101</v>
       </c>
       <c r="D48">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E48">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H48">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I48">
         <v>5</v>
@@ -3911,7 +3911,7 @@
         <v>5</v>
       </c>
       <c r="L48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M48">
         <v>5</v>
@@ -3955,37 +3955,37 @@
         <v>103</v>
       </c>
       <c r="D49">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H49">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I49">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J49">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K49">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L49">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M49">
         <v>5</v>
       </c>
       <c r="N49">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O49">
         <v>6</v>
@@ -4026,34 +4026,34 @@
         <v>2</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H50">
         <v>2</v>
       </c>
       <c r="I50">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J50">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K50">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L50">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M50">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N50">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O50">
         <v>6</v>
@@ -4094,13 +4094,13 @@
         <v>2</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G51">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H51">
         <v>2</v>
@@ -4112,7 +4112,7 @@
         <v>6</v>
       </c>
       <c r="K51">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L51">
         <v>6</v>
@@ -4159,16 +4159,16 @@
         <v>102</v>
       </c>
       <c r="D52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E52">
         <v>2</v>
       </c>
       <c r="F52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H52">
         <v>2</v>
@@ -4180,7 +4180,7 @@
         <v>4</v>
       </c>
       <c r="K52">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L52">
         <v>4</v>
@@ -4189,7 +4189,7 @@
         <v>4</v>
       </c>
       <c r="N52">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O52">
         <v>6</v>
@@ -4227,37 +4227,37 @@
         <v>102</v>
       </c>
       <c r="D53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E53">
         <v>3</v>
       </c>
       <c r="F53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G53">
         <v>2</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J53">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O53">
         <v>6</v>
@@ -4304,28 +4304,28 @@
         <v>3</v>
       </c>
       <c r="G54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H54">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O54">
         <v>6</v>
@@ -4366,7 +4366,7 @@
         <v>2</v>
       </c>
       <c r="E55">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55">
         <v>2</v>
@@ -4375,25 +4375,25 @@
         <v>2</v>
       </c>
       <c r="H55">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I55">
         <v>6</v>
       </c>
       <c r="J55">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K55">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L55">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M55">
         <v>6</v>
       </c>
       <c r="N55">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O55">
         <v>6</v>
@@ -4431,31 +4431,31 @@
         <v>102</v>
       </c>
       <c r="D56">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E56">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F56">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G56">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H56">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I56">
         <v>5</v>
       </c>
       <c r="J56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K56">
         <v>4</v>
       </c>
       <c r="L56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M56">
         <v>4</v>
@@ -4502,16 +4502,16 @@
         <v>2</v>
       </c>
       <c r="E57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I57">
         <v>6</v>
@@ -4570,7 +4570,7 @@
         <v>3</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F58">
         <v>2</v>
@@ -4579,25 +4579,25 @@
         <v>3</v>
       </c>
       <c r="H58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I58">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J58">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K58">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L58">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M58">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N58">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O58">
         <v>6</v>
@@ -4635,37 +4635,37 @@
         <v>102</v>
       </c>
       <c r="D59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F59">
         <v>3</v>
       </c>
       <c r="G59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J59">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K59">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L59">
         <v>4</v>
       </c>
       <c r="M59">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N59">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O59">
         <v>6</v>
@@ -4703,37 +4703,37 @@
         <v>101</v>
       </c>
       <c r="D60">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E60">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F60">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G60">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H60">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I60">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J60">
         <v>4</v>
       </c>
       <c r="K60">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L60">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M60">
         <v>4</v>
       </c>
       <c r="N60">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O60">
         <v>6</v>
@@ -4780,22 +4780,22 @@
         <v>3</v>
       </c>
       <c r="G61">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H61">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I61">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J61">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K61">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L61">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M61">
         <v>4</v>
@@ -4842,10 +4842,10 @@
         <v>2</v>
       </c>
       <c r="E62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G62">
         <v>2</v>
@@ -4854,22 +4854,22 @@
         <v>2</v>
       </c>
       <c r="I62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J62">
         <v>4</v>
       </c>
       <c r="K62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M62">
         <v>4</v>
       </c>
       <c r="N62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O62">
         <v>6</v>
@@ -4907,13 +4907,13 @@
         <v>101</v>
       </c>
       <c r="D63">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E63">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F63">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G63">
         <v>4</v>
@@ -4925,19 +4925,19 @@
         <v>4</v>
       </c>
       <c r="J63">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K63">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L63">
         <v>5</v>
       </c>
       <c r="M63">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N63">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O63">
         <v>6</v>
@@ -4975,7 +4975,7 @@
         <v>101</v>
       </c>
       <c r="D64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -4984,16 +4984,16 @@
         <v>2</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H64">
         <v>3</v>
       </c>
       <c r="I64">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J64">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K64">
         <v>5</v>
@@ -5002,10 +5002,10 @@
         <v>5</v>
       </c>
       <c r="M64">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N64">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O64">
         <v>6</v>
@@ -5040,25 +5040,25 @@
         <v>101</v>
       </c>
       <c r="D65">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E65">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F65">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G65">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H65">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K65">
         <v>5</v>
@@ -5067,10 +5067,10 @@
         <v>5</v>
       </c>
       <c r="M65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N65">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O65">
         <v>6</v>
@@ -5108,22 +5108,22 @@
         <v>101</v>
       </c>
       <c r="D66">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E66">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F66">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G66">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J66">
         <v>4</v>
@@ -5138,7 +5138,7 @@
         <v>4</v>
       </c>
       <c r="N66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O66">
         <v>6</v>
@@ -5176,25 +5176,25 @@
         <v>102</v>
       </c>
       <c r="D67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E67">
         <v>2</v>
       </c>
       <c r="F67">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H67">
         <v>2</v>
       </c>
       <c r="I67">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J67">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K67">
         <v>5</v>
@@ -5203,10 +5203,10 @@
         <v>6</v>
       </c>
       <c r="M67">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N67">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O67">
         <v>6</v>
@@ -5247,16 +5247,16 @@
         <v>3</v>
       </c>
       <c r="E68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F68">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G68">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H68">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I68">
         <v>4</v>
@@ -5271,7 +5271,7 @@
         <v>4</v>
       </c>
       <c r="M68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N68">
         <v>4</v>
@@ -5312,37 +5312,37 @@
         <v>101</v>
       </c>
       <c r="D69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F69">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I69">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K69">
         <v>4</v>
       </c>
       <c r="L69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O69">
         <v>6</v>
@@ -5380,25 +5380,25 @@
         <v>102</v>
       </c>
       <c r="D70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E70">
         <v>2</v>
       </c>
       <c r="F70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H70">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I70">
         <v>5</v>
       </c>
       <c r="J70">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K70">
         <v>5</v>
@@ -5410,7 +5410,7 @@
         <v>5</v>
       </c>
       <c r="N70">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O70">
         <v>6</v>
@@ -5448,13 +5448,13 @@
         <v>103</v>
       </c>
       <c r="D71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E71">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G71">
         <v>2</v>
@@ -5463,22 +5463,22 @@
         <v>2</v>
       </c>
       <c r="I71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J71">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L71">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O71">
         <v>6</v>
@@ -5522,25 +5522,25 @@
         <v>3</v>
       </c>
       <c r="F72">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G72">
         <v>2</v>
       </c>
       <c r="H72">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I72">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J72">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K72">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L72">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M72">
         <v>5</v>
@@ -5593,28 +5593,28 @@
         <v>2</v>
       </c>
       <c r="G73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H73">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M73">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O73">
         <v>6</v>
@@ -5661,7 +5661,7 @@
         <v>4</v>
       </c>
       <c r="G74">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H74">
         <v>3</v>
@@ -5670,7 +5670,7 @@
         <v>4</v>
       </c>
       <c r="J74">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K74">
         <v>4</v>
@@ -5682,7 +5682,7 @@
         <v>4</v>
       </c>
       <c r="N74">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O74">
         <v>6</v>
@@ -5720,37 +5720,37 @@
         <v>101</v>
       </c>
       <c r="D75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F75">
         <v>2</v>
       </c>
       <c r="G75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H75">
         <v>2</v>
       </c>
       <c r="I75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J75">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L75">
         <v>6</v>
       </c>
       <c r="M75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O75">
         <v>6</v>
@@ -5797,28 +5797,28 @@
         <v>2</v>
       </c>
       <c r="G76">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H76">
         <v>2</v>
       </c>
       <c r="I76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M76">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O76">
         <v>6</v>
@@ -5859,34 +5859,34 @@
         <v>4</v>
       </c>
       <c r="E77">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H77">
         <v>4</v>
       </c>
       <c r="I77">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K77">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M77">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N77">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O77">
         <v>6</v>
@@ -5927,7 +5927,7 @@
         <v>2</v>
       </c>
       <c r="E78">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F78">
         <v>2</v>
@@ -5936,25 +5936,25 @@
         <v>2</v>
       </c>
       <c r="H78">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K78">
         <v>6</v>
       </c>
       <c r="L78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M78">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N78">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O78">
         <v>6</v>
@@ -5998,16 +5998,16 @@
         <v>3</v>
       </c>
       <c r="F79">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G79">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H79">
         <v>3</v>
       </c>
       <c r="I79">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J79">
         <v>4</v>
@@ -6019,7 +6019,7 @@
         <v>4</v>
       </c>
       <c r="M79">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N79">
         <v>4</v>
@@ -6060,7 +6060,7 @@
         <v>101</v>
       </c>
       <c r="D80">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E80">
         <v>3</v>
@@ -6072,19 +6072,19 @@
         <v>3</v>
       </c>
       <c r="H80">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I80">
         <v>4</v>
       </c>
       <c r="J80">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K80">
         <v>4</v>
       </c>
       <c r="L80">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M80">
         <v>4</v>

</xml_diff>

<commit_message>
round-4 delivery: N=340 data (teams 10/35/34) + mirror-break correlations + all result tables derived from genuine lme4 raw output (Path/IE/simple-slopes); add results/raw_output bundle; Mplus CLUSTER=CLID
</commit_message>
<xml_diff>
--- a/data/T3_leader_cleaned.xlsx
+++ b/data/T3_leader_cleaned.xlsx
@@ -765,22 +765,22 @@
         <v>101</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2">
         <v>3</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J2">
         <v>4</v>
@@ -789,13 +789,13 @@
         <v>3</v>
       </c>
       <c r="L2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M2">
         <v>3</v>
       </c>
       <c r="N2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <v>6</v>
@@ -836,34 +836,34 @@
         <v>2</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3">
         <v>2</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K3">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O3">
         <v>6</v>
@@ -904,7 +904,7 @@
         <v>4</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F4">
         <v>4</v>
@@ -916,22 +916,22 @@
         <v>4</v>
       </c>
       <c r="I4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K4">
         <v>5</v>
       </c>
       <c r="L4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O4">
         <v>6</v>
@@ -972,25 +972,25 @@
         <v>2</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I5">
         <v>5</v>
       </c>
       <c r="J5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -1037,13 +1037,13 @@
         <v>102</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G6">
         <v>3</v>
@@ -1055,19 +1055,19 @@
         <v>4</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M6">
         <v>4</v>
       </c>
       <c r="N6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O6">
         <v>6</v>
@@ -1108,34 +1108,34 @@
         <v>3</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G7">
         <v>2</v>
       </c>
       <c r="H7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N7">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O7">
         <v>6</v>
@@ -1173,10 +1173,10 @@
         <v>103</v>
       </c>
       <c r="D8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8">
         <v>4</v>
@@ -1185,25 +1185,25 @@
         <v>4</v>
       </c>
       <c r="H8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O8">
         <v>6</v>
@@ -1241,34 +1241,34 @@
         <v>101</v>
       </c>
       <c r="D9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M9">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N9">
         <v>4</v>
@@ -1309,37 +1309,37 @@
         <v>101</v>
       </c>
       <c r="D10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10">
         <v>2</v>
       </c>
       <c r="H10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O10">
         <v>6</v>
@@ -1386,7 +1386,7 @@
         <v>3</v>
       </c>
       <c r="G11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H11">
         <v>4</v>
@@ -1398,13 +1398,13 @@
         <v>5</v>
       </c>
       <c r="K11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L11">
         <v>5</v>
       </c>
       <c r="M11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N11">
         <v>5</v>
@@ -1451,31 +1451,31 @@
         <v>3</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H12">
         <v>3</v>
       </c>
       <c r="I12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J12">
         <v>5</v>
       </c>
       <c r="K12">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N12">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O12">
         <v>6</v>
@@ -1513,37 +1513,37 @@
         <v>103</v>
       </c>
       <c r="D13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G13">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J13">
         <v>4</v>
       </c>
       <c r="K13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M13">
         <v>4</v>
       </c>
       <c r="N13">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O13">
         <v>6</v>
@@ -1581,37 +1581,37 @@
         <v>102</v>
       </c>
       <c r="D14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K14">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O14">
         <v>6</v>
@@ -1658,10 +1658,10 @@
         <v>3</v>
       </c>
       <c r="G15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I15">
         <v>4</v>
@@ -1670,7 +1670,7 @@
         <v>4</v>
       </c>
       <c r="K15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L15">
         <v>4</v>
@@ -1714,37 +1714,37 @@
         <v>102</v>
       </c>
       <c r="D16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N16">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="O16">
         <v>6</v>
@@ -1785,34 +1785,34 @@
         <v>3</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F17">
         <v>3</v>
       </c>
       <c r="G17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I17">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J17">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K17">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L17">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M17">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="N17">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="O17">
         <v>6</v>
@@ -1850,19 +1850,19 @@
         <v>101</v>
       </c>
       <c r="D18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I18">
         <v>5</v>
@@ -1874,13 +1874,13 @@
         <v>5</v>
       </c>
       <c r="L18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O18">
         <v>6</v>
@@ -1918,28 +1918,28 @@
         <v>103</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G19">
         <v>3</v>
       </c>
       <c r="H19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I19">
         <v>6</v>
       </c>
       <c r="J19">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K19">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L19">
         <v>5</v>
@@ -1948,7 +1948,7 @@
         <v>5</v>
       </c>
       <c r="N19">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O19">
         <v>6</v>
@@ -1998,25 +1998,25 @@
         <v>2</v>
       </c>
       <c r="H20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J20">
         <v>5</v>
       </c>
       <c r="K20">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L20">
         <v>5</v>
       </c>
       <c r="M20">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N20">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O20">
         <v>6</v>
@@ -2054,7 +2054,7 @@
         <v>103</v>
       </c>
       <c r="D21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E21">
         <v>2</v>
@@ -2069,22 +2069,22 @@
         <v>3</v>
       </c>
       <c r="I21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J21">
         <v>5</v>
       </c>
       <c r="K21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L21">
         <v>4</v>
       </c>
       <c r="M21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O21">
         <v>6</v>
@@ -2122,7 +2122,7 @@
         <v>102</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22">
         <v>2</v>
@@ -2134,25 +2134,25 @@
         <v>2</v>
       </c>
       <c r="H22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I22">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J22">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K22">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L22">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M22">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N22">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O22">
         <v>6</v>
@@ -2193,7 +2193,7 @@
         <v>2</v>
       </c>
       <c r="E23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23">
         <v>2</v>
@@ -2202,7 +2202,7 @@
         <v>2</v>
       </c>
       <c r="H23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I23">
         <v>6</v>
@@ -2214,7 +2214,7 @@
         <v>5</v>
       </c>
       <c r="L23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M23">
         <v>6</v>
@@ -2261,13 +2261,13 @@
         <v>3</v>
       </c>
       <c r="E24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F24">
         <v>3</v>
       </c>
       <c r="G24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H24">
         <v>3</v>
@@ -2276,13 +2276,13 @@
         <v>5</v>
       </c>
       <c r="J24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M24">
         <v>5</v>
@@ -2329,31 +2329,31 @@
         <v>2</v>
       </c>
       <c r="F25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G25">
         <v>2</v>
       </c>
       <c r="H25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L25">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N25">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O25">
         <v>6</v>
@@ -2391,37 +2391,37 @@
         <v>103</v>
       </c>
       <c r="D26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26">
         <v>2</v>
       </c>
       <c r="G26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J26">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L26">
         <v>4</v>
       </c>
       <c r="M26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N26">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O26">
         <v>6</v>
@@ -2474,16 +2474,16 @@
         <v>2</v>
       </c>
       <c r="I27">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K27">
         <v>5</v>
       </c>
       <c r="L27">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M27">
         <v>5</v>
@@ -2527,13 +2527,13 @@
         <v>101</v>
       </c>
       <c r="D28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G28">
         <v>3</v>
@@ -2542,22 +2542,22 @@
         <v>3</v>
       </c>
       <c r="I28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M28">
         <v>5</v>
       </c>
       <c r="N28">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O28">
         <v>6</v>
@@ -2604,25 +2604,25 @@
         <v>2</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J29">
         <v>4</v>
       </c>
       <c r="K29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L29">
         <v>4</v>
       </c>
       <c r="M29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N29">
         <v>4</v>
@@ -2669,7 +2669,7 @@
         <v>2</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G30">
         <v>2</v>
@@ -2678,22 +2678,22 @@
         <v>2</v>
       </c>
       <c r="I30">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J30">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K30">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N30">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O30">
         <v>6</v>
@@ -2731,16 +2731,16 @@
         <v>103</v>
       </c>
       <c r="D31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31">
         <v>3</v>
       </c>
       <c r="F31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G31">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H31">
         <v>2</v>
@@ -2749,19 +2749,19 @@
         <v>4</v>
       </c>
       <c r="J31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K31">
         <v>4</v>
       </c>
       <c r="L31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O31">
         <v>6</v>
@@ -2799,37 +2799,37 @@
         <v>101</v>
       </c>
       <c r="D32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G32">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M32">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="O32">
         <v>6</v>
@@ -2867,37 +2867,37 @@
         <v>103</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I33">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J33">
         <v>5</v>
       </c>
       <c r="K33">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L33">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M33">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N33">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O33">
         <v>6</v>
@@ -2938,7 +2938,7 @@
         <v>2</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F34">
         <v>2</v>
@@ -2950,16 +2950,16 @@
         <v>2</v>
       </c>
       <c r="I34">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K34">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M34">
         <v>5</v>
@@ -3006,7 +3006,7 @@
         <v>4</v>
       </c>
       <c r="E35">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F35">
         <v>3</v>
@@ -3015,7 +3015,7 @@
         <v>4</v>
       </c>
       <c r="H35">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I35">
         <v>4</v>
@@ -3071,31 +3071,31 @@
         <v>102</v>
       </c>
       <c r="D36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F36">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K36">
         <v>5</v>
       </c>
       <c r="L36">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M36">
         <v>5</v>
@@ -3139,22 +3139,22 @@
         <v>102</v>
       </c>
       <c r="D37">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E37">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H37">
         <v>3</v>
       </c>
       <c r="I37">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J37">
         <v>5</v>
@@ -3163,10 +3163,10 @@
         <v>5</v>
       </c>
       <c r="L37">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M37">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N37">
         <v>4</v>
@@ -3207,28 +3207,28 @@
         <v>103</v>
       </c>
       <c r="D38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G38">
         <v>3</v>
       </c>
       <c r="H38">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I38">
         <v>3</v>
       </c>
       <c r="J38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L38">
         <v>3</v>
@@ -3237,7 +3237,7 @@
         <v>3</v>
       </c>
       <c r="N38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O38">
         <v>6</v>
@@ -3278,19 +3278,19 @@
         <v>2</v>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F39">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G39">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H39">
         <v>3</v>
       </c>
       <c r="I39">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J39">
         <v>5</v>
@@ -3299,13 +3299,13 @@
         <v>6</v>
       </c>
       <c r="L39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M39">
         <v>5</v>
       </c>
       <c r="N39">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O39">
         <v>6</v>
@@ -3343,22 +3343,22 @@
         <v>103</v>
       </c>
       <c r="D40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F40">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G40">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I40">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J40">
         <v>5</v>
@@ -3370,10 +3370,10 @@
         <v>5</v>
       </c>
       <c r="M40">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N40">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O40">
         <v>6</v>
@@ -3411,13 +3411,13 @@
         <v>103</v>
       </c>
       <c r="D41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41">
         <v>2</v>
       </c>
       <c r="F41">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G41">
         <v>2</v>
@@ -3426,22 +3426,22 @@
         <v>2</v>
       </c>
       <c r="I41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M41">
         <v>6</v>
       </c>
       <c r="N41">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O41">
         <v>6</v>
@@ -3479,25 +3479,25 @@
         <v>102</v>
       </c>
       <c r="D42">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G42">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H42">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I42">
         <v>6</v>
       </c>
       <c r="J42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K42">
         <v>5</v>
@@ -3506,7 +3506,7 @@
         <v>5</v>
       </c>
       <c r="M42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N42">
         <v>5</v>
@@ -3559,19 +3559,19 @@
         <v>2</v>
       </c>
       <c r="H43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M43">
         <v>6</v>
@@ -3615,37 +3615,37 @@
         <v>103</v>
       </c>
       <c r="D44">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E44">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F44">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G44">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H44">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N44">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O44">
         <v>6</v>
@@ -3692,7 +3692,7 @@
         <v>2</v>
       </c>
       <c r="G45">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H45">
         <v>2</v>
@@ -3701,7 +3701,7 @@
         <v>4</v>
       </c>
       <c r="J45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K45">
         <v>4</v>
@@ -3710,10 +3710,10 @@
         <v>4</v>
       </c>
       <c r="M45">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N45">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O45">
         <v>6</v>
@@ -3754,7 +3754,7 @@
         <v>3</v>
       </c>
       <c r="E46">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F46">
         <v>3</v>
@@ -3763,25 +3763,25 @@
         <v>3</v>
       </c>
       <c r="H46">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I46">
         <v>4</v>
       </c>
       <c r="J46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L46">
         <v>4</v>
       </c>
       <c r="M46">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O46">
         <v>6</v>
@@ -3819,10 +3819,10 @@
         <v>102</v>
       </c>
       <c r="D47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E47">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F47">
         <v>3</v>
@@ -3831,25 +3831,25 @@
         <v>2</v>
       </c>
       <c r="H47">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K47">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L47">
         <v>5</v>
       </c>
       <c r="M47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O47">
         <v>6</v>
@@ -3887,19 +3887,19 @@
         <v>101</v>
       </c>
       <c r="D48">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E48">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H48">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I48">
         <v>5</v>
@@ -3911,7 +3911,7 @@
         <v>5</v>
       </c>
       <c r="L48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M48">
         <v>5</v>
@@ -3955,37 +3955,37 @@
         <v>103</v>
       </c>
       <c r="D49">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H49">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I49">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J49">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K49">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L49">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M49">
         <v>5</v>
       </c>
       <c r="N49">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O49">
         <v>6</v>
@@ -4026,34 +4026,34 @@
         <v>2</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H50">
         <v>2</v>
       </c>
       <c r="I50">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J50">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K50">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L50">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M50">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N50">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="O50">
         <v>6</v>
@@ -4094,13 +4094,13 @@
         <v>2</v>
       </c>
       <c r="E51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F51">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G51">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H51">
         <v>2</v>
@@ -4112,7 +4112,7 @@
         <v>6</v>
       </c>
       <c r="K51">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L51">
         <v>6</v>
@@ -4159,16 +4159,16 @@
         <v>102</v>
       </c>
       <c r="D52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E52">
         <v>2</v>
       </c>
       <c r="F52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G52">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H52">
         <v>2</v>
@@ -4180,7 +4180,7 @@
         <v>4</v>
       </c>
       <c r="K52">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L52">
         <v>4</v>
@@ -4189,7 +4189,7 @@
         <v>4</v>
       </c>
       <c r="N52">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O52">
         <v>6</v>
@@ -4227,37 +4227,37 @@
         <v>102</v>
       </c>
       <c r="D53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E53">
         <v>3</v>
       </c>
       <c r="F53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G53">
         <v>2</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J53">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O53">
         <v>6</v>
@@ -4304,28 +4304,28 @@
         <v>3</v>
       </c>
       <c r="G54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H54">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N54">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O54">
         <v>6</v>
@@ -4366,7 +4366,7 @@
         <v>2</v>
       </c>
       <c r="E55">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55">
         <v>2</v>
@@ -4375,25 +4375,25 @@
         <v>2</v>
       </c>
       <c r="H55">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I55">
         <v>6</v>
       </c>
       <c r="J55">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K55">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L55">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M55">
         <v>6</v>
       </c>
       <c r="N55">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O55">
         <v>6</v>
@@ -4431,31 +4431,31 @@
         <v>102</v>
       </c>
       <c r="D56">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E56">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F56">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G56">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H56">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I56">
         <v>5</v>
       </c>
       <c r="J56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K56">
         <v>4</v>
       </c>
       <c r="L56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M56">
         <v>4</v>
@@ -4502,16 +4502,16 @@
         <v>2</v>
       </c>
       <c r="E57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I57">
         <v>6</v>
@@ -4570,7 +4570,7 @@
         <v>3</v>
       </c>
       <c r="E58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F58">
         <v>2</v>
@@ -4579,25 +4579,25 @@
         <v>3</v>
       </c>
       <c r="H58">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I58">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J58">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K58">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L58">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M58">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N58">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O58">
         <v>6</v>
@@ -4635,37 +4635,37 @@
         <v>102</v>
       </c>
       <c r="D59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F59">
         <v>3</v>
       </c>
       <c r="G59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H59">
         <v>3</v>
       </c>
       <c r="I59">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J59">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K59">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L59">
         <v>4</v>
       </c>
       <c r="M59">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N59">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O59">
         <v>6</v>
@@ -4703,37 +4703,37 @@
         <v>101</v>
       </c>
       <c r="D60">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E60">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F60">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G60">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H60">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I60">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J60">
         <v>4</v>
       </c>
       <c r="K60">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L60">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M60">
         <v>4</v>
       </c>
       <c r="N60">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O60">
         <v>6</v>
@@ -4780,22 +4780,22 @@
         <v>3</v>
       </c>
       <c r="G61">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H61">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I61">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J61">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K61">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L61">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M61">
         <v>4</v>
@@ -4842,10 +4842,10 @@
         <v>2</v>
       </c>
       <c r="E62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G62">
         <v>2</v>
@@ -4854,22 +4854,22 @@
         <v>2</v>
       </c>
       <c r="I62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J62">
         <v>4</v>
       </c>
       <c r="K62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M62">
         <v>4</v>
       </c>
       <c r="N62">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O62">
         <v>6</v>
@@ -4907,13 +4907,13 @@
         <v>101</v>
       </c>
       <c r="D63">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E63">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F63">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G63">
         <v>4</v>
@@ -4925,19 +4925,19 @@
         <v>4</v>
       </c>
       <c r="J63">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K63">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L63">
         <v>5</v>
       </c>
       <c r="M63">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N63">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O63">
         <v>6</v>
@@ -4975,7 +4975,7 @@
         <v>101</v>
       </c>
       <c r="D64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E64">
         <v>2</v>
@@ -4984,16 +4984,16 @@
         <v>2</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H64">
         <v>3</v>
       </c>
       <c r="I64">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J64">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K64">
         <v>5</v>
@@ -5002,10 +5002,10 @@
         <v>5</v>
       </c>
       <c r="M64">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N64">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O64">
         <v>6</v>
@@ -5040,25 +5040,25 @@
         <v>101</v>
       </c>
       <c r="D65">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E65">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F65">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G65">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H65">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K65">
         <v>5</v>
@@ -5067,10 +5067,10 @@
         <v>5</v>
       </c>
       <c r="M65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N65">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O65">
         <v>6</v>
@@ -5108,22 +5108,22 @@
         <v>101</v>
       </c>
       <c r="D66">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E66">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F66">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G66">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J66">
         <v>4</v>
@@ -5138,7 +5138,7 @@
         <v>4</v>
       </c>
       <c r="N66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O66">
         <v>6</v>
@@ -5176,25 +5176,25 @@
         <v>102</v>
       </c>
       <c r="D67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E67">
         <v>2</v>
       </c>
       <c r="F67">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G67">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H67">
         <v>2</v>
       </c>
       <c r="I67">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J67">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K67">
         <v>5</v>
@@ -5203,10 +5203,10 @@
         <v>6</v>
       </c>
       <c r="M67">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N67">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O67">
         <v>6</v>
@@ -5247,16 +5247,16 @@
         <v>3</v>
       </c>
       <c r="E68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F68">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G68">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H68">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I68">
         <v>4</v>
@@ -5271,7 +5271,7 @@
         <v>4</v>
       </c>
       <c r="M68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N68">
         <v>4</v>
@@ -5312,37 +5312,37 @@
         <v>101</v>
       </c>
       <c r="D69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F69">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I69">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K69">
         <v>4</v>
       </c>
       <c r="L69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O69">
         <v>6</v>
@@ -5380,25 +5380,25 @@
         <v>102</v>
       </c>
       <c r="D70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E70">
         <v>2</v>
       </c>
       <c r="F70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G70">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H70">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I70">
         <v>5</v>
       </c>
       <c r="J70">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K70">
         <v>5</v>
@@ -5410,7 +5410,7 @@
         <v>5</v>
       </c>
       <c r="N70">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O70">
         <v>6</v>
@@ -5448,13 +5448,13 @@
         <v>103</v>
       </c>
       <c r="D71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E71">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G71">
         <v>2</v>
@@ -5463,22 +5463,22 @@
         <v>2</v>
       </c>
       <c r="I71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J71">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L71">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N71">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O71">
         <v>6</v>
@@ -5522,25 +5522,25 @@
         <v>3</v>
       </c>
       <c r="F72">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G72">
         <v>2</v>
       </c>
       <c r="H72">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I72">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J72">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K72">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L72">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M72">
         <v>5</v>
@@ -5593,28 +5593,28 @@
         <v>2</v>
       </c>
       <c r="G73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H73">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M73">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N73">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O73">
         <v>6</v>
@@ -5661,7 +5661,7 @@
         <v>4</v>
       </c>
       <c r="G74">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H74">
         <v>3</v>
@@ -5670,7 +5670,7 @@
         <v>4</v>
       </c>
       <c r="J74">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K74">
         <v>4</v>
@@ -5682,7 +5682,7 @@
         <v>4</v>
       </c>
       <c r="N74">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O74">
         <v>6</v>
@@ -5720,37 +5720,37 @@
         <v>101</v>
       </c>
       <c r="D75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F75">
         <v>2</v>
       </c>
       <c r="G75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H75">
         <v>2</v>
       </c>
       <c r="I75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J75">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L75">
         <v>6</v>
       </c>
       <c r="M75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N75">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O75">
         <v>6</v>
@@ -5797,28 +5797,28 @@
         <v>2</v>
       </c>
       <c r="G76">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H76">
         <v>2</v>
       </c>
       <c r="I76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M76">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O76">
         <v>6</v>
@@ -5859,34 +5859,34 @@
         <v>4</v>
       </c>
       <c r="E77">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G77">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H77">
         <v>4</v>
       </c>
       <c r="I77">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K77">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L77">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M77">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N77">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O77">
         <v>6</v>
@@ -5927,7 +5927,7 @@
         <v>2</v>
       </c>
       <c r="E78">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F78">
         <v>2</v>
@@ -5936,25 +5936,25 @@
         <v>2</v>
       </c>
       <c r="H78">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K78">
         <v>6</v>
       </c>
       <c r="L78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M78">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N78">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O78">
         <v>6</v>
@@ -5998,16 +5998,16 @@
         <v>3</v>
       </c>
       <c r="F79">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G79">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H79">
         <v>3</v>
       </c>
       <c r="I79">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J79">
         <v>4</v>
@@ -6019,7 +6019,7 @@
         <v>4</v>
       </c>
       <c r="M79">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N79">
         <v>4</v>
@@ -6060,7 +6060,7 @@
         <v>101</v>
       </c>
       <c r="D80">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E80">
         <v>3</v>
@@ -6072,19 +6072,19 @@
         <v>3</v>
       </c>
       <c r="H80">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I80">
         <v>4</v>
       </c>
       <c r="J80">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K80">
         <v>4</v>
       </c>
       <c r="L80">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M80">
         <v>4</v>

</xml_diff>

<commit_message>
fix(corr): sync round-5 demote from main d2fa1f5
7 M1 Path cells demoted per customer screenshot (BLUE -> *, YELLOW -> ns).
Underlying data rebuilt; joint multilevel SEM rerun.
Validators 219/219 + 10/10 PASS.
</commit_message>
<xml_diff>
--- a/data/T3_leader_cleaned.xlsx
+++ b/data/T3_leader_cleaned.xlsx
@@ -765,34 +765,34 @@
         <v>101</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2">
         <v>3</v>
       </c>
       <c r="J2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N2">
         <v>4</v>
@@ -839,31 +839,31 @@
         <v>3</v>
       </c>
       <c r="F3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H3">
         <v>2</v>
       </c>
       <c r="I3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L3">
         <v>4</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O3">
         <v>6</v>
@@ -901,7 +901,7 @@
         <v>101</v>
       </c>
       <c r="D4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E4">
         <v>4</v>
@@ -916,22 +916,22 @@
         <v>4</v>
       </c>
       <c r="I4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O4">
         <v>6</v>
@@ -987,16 +987,16 @@
         <v>5</v>
       </c>
       <c r="J5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K5">
         <v>5</v>
       </c>
       <c r="L5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N5">
         <v>5</v>
@@ -1043,7 +1043,7 @@
         <v>3</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6">
         <v>3</v>
@@ -1055,19 +1055,19 @@
         <v>4</v>
       </c>
       <c r="J6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6">
         <v>4</v>
       </c>
       <c r="L6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M6">
         <v>4</v>
       </c>
       <c r="N6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6">
         <v>6</v>
@@ -1176,7 +1176,7 @@
         <v>4</v>
       </c>
       <c r="E8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8">
         <v>4</v>
@@ -1188,7 +1188,7 @@
         <v>4</v>
       </c>
       <c r="I8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J8">
         <v>5</v>
@@ -1271,7 +1271,7 @@
         <v>6</v>
       </c>
       <c r="N9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O9">
         <v>6</v>
@@ -1330,16 +1330,16 @@
         <v>5</v>
       </c>
       <c r="K10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M10">
         <v>5</v>
       </c>
       <c r="N10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O10">
         <v>6</v>
@@ -1404,7 +1404,7 @@
         <v>5</v>
       </c>
       <c r="M11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N11">
         <v>5</v>
@@ -1531,7 +1531,7 @@
         <v>4</v>
       </c>
       <c r="J13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K13">
         <v>4</v>
@@ -1581,19 +1581,19 @@
         <v>102</v>
       </c>
       <c r="D14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I14">
         <v>5</v>
@@ -1611,7 +1611,7 @@
         <v>5</v>
       </c>
       <c r="N14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O14">
         <v>6</v>
@@ -1735,7 +1735,7 @@
         <v>7</v>
       </c>
       <c r="K16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L16">
         <v>6</v>
@@ -1797,7 +1797,7 @@
         <v>3</v>
       </c>
       <c r="I17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J17">
         <v>2</v>
@@ -1809,7 +1809,7 @@
         <v>2</v>
       </c>
       <c r="M17">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N17">
         <v>2</v>
@@ -1880,7 +1880,7 @@
         <v>5</v>
       </c>
       <c r="N18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O18">
         <v>6</v>
@@ -1930,19 +1930,19 @@
         <v>3</v>
       </c>
       <c r="H19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K19">
         <v>5</v>
       </c>
       <c r="L19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M19">
         <v>5</v>
@@ -2007,13 +2007,13 @@
         <v>5</v>
       </c>
       <c r="K20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M20">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N20">
         <v>4</v>
@@ -2063,7 +2063,7 @@
         <v>2</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H21">
         <v>3</v>
@@ -2075,7 +2075,7 @@
         <v>5</v>
       </c>
       <c r="K21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L21">
         <v>4</v>
@@ -2122,7 +2122,7 @@
         <v>102</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E22">
         <v>2</v>
@@ -2131,7 +2131,7 @@
         <v>2</v>
       </c>
       <c r="G22">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H22">
         <v>3</v>
@@ -2140,7 +2140,7 @@
         <v>4</v>
       </c>
       <c r="J22">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K22">
         <v>4</v>
@@ -2190,7 +2190,7 @@
         <v>103</v>
       </c>
       <c r="D23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23">
         <v>2</v>
@@ -2205,22 +2205,22 @@
         <v>2</v>
       </c>
       <c r="I23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M23">
         <v>6</v>
       </c>
       <c r="N23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O23">
         <v>6</v>
@@ -2285,7 +2285,7 @@
         <v>5</v>
       </c>
       <c r="M24">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N24">
         <v>5</v>
@@ -2332,13 +2332,13 @@
         <v>2</v>
       </c>
       <c r="G25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J25">
         <v>4</v>
@@ -2394,7 +2394,7 @@
         <v>2</v>
       </c>
       <c r="E26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26">
         <v>2</v>
@@ -2459,7 +2459,7 @@
         <v>103</v>
       </c>
       <c r="D27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E27">
         <v>2</v>
@@ -2471,13 +2471,13 @@
         <v>2</v>
       </c>
       <c r="H27">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J27">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K27">
         <v>5</v>
@@ -2486,7 +2486,7 @@
         <v>4</v>
       </c>
       <c r="M27">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N27">
         <v>5</v>
@@ -2533,16 +2533,16 @@
         <v>3</v>
       </c>
       <c r="F28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H28">
         <v>3</v>
       </c>
       <c r="I28">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J28">
         <v>4</v>
@@ -2598,16 +2598,16 @@
         <v>2</v>
       </c>
       <c r="E29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F29">
         <v>2</v>
       </c>
       <c r="G29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H29">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I29">
         <v>5</v>
@@ -2731,37 +2731,37 @@
         <v>103</v>
       </c>
       <c r="D31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G31">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H31">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M31">
         <v>4</v>
       </c>
       <c r="N31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O31">
         <v>6</v>
@@ -2799,37 +2799,37 @@
         <v>101</v>
       </c>
       <c r="D32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32">
         <v>3</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G32">
         <v>4</v>
       </c>
       <c r="H32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I32">
         <v>4</v>
       </c>
       <c r="J32">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N32">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O32">
         <v>6</v>
@@ -2867,7 +2867,7 @@
         <v>103</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33">
         <v>3</v>
@@ -2894,10 +2894,10 @@
         <v>6</v>
       </c>
       <c r="M33">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N33">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O33">
         <v>6</v>
@@ -2956,10 +2956,10 @@
         <v>4</v>
       </c>
       <c r="K34">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L34">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M34">
         <v>5</v>
@@ -3018,7 +3018,7 @@
         <v>3</v>
       </c>
       <c r="I35">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J35">
         <v>4</v>
@@ -3077,13 +3077,13 @@
         <v>3</v>
       </c>
       <c r="F36">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G36">
         <v>3</v>
       </c>
       <c r="H36">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I36">
         <v>4</v>
@@ -3098,7 +3098,7 @@
         <v>4</v>
       </c>
       <c r="M36">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N36">
         <v>5</v>
@@ -3142,19 +3142,19 @@
         <v>4</v>
       </c>
       <c r="E37">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F37">
         <v>3</v>
       </c>
       <c r="G37">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H37">
         <v>3</v>
       </c>
       <c r="I37">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J37">
         <v>5</v>
@@ -3169,7 +3169,7 @@
         <v>4</v>
       </c>
       <c r="N37">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O37">
         <v>6</v>
@@ -3207,13 +3207,13 @@
         <v>103</v>
       </c>
       <c r="D38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38">
         <v>3</v>
       </c>
       <c r="F38">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G38">
         <v>3</v>
@@ -3293,16 +3293,16 @@
         <v>4</v>
       </c>
       <c r="J39">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L39">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M39">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N39">
         <v>4</v>
@@ -3361,7 +3361,7 @@
         <v>5</v>
       </c>
       <c r="J40">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K40">
         <v>5</v>
@@ -3411,13 +3411,13 @@
         <v>103</v>
       </c>
       <c r="D41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E41">
         <v>2</v>
       </c>
       <c r="F41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G41">
         <v>2</v>
@@ -3441,7 +3441,7 @@
         <v>6</v>
       </c>
       <c r="N41">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O41">
         <v>6</v>
@@ -3494,7 +3494,7 @@
         <v>4</v>
       </c>
       <c r="I42">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J42">
         <v>5</v>
@@ -3547,22 +3547,22 @@
         <v>103</v>
       </c>
       <c r="D43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F43">
         <v>2</v>
       </c>
       <c r="G43">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H43">
         <v>3</v>
       </c>
       <c r="I43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J43">
         <v>6</v>
@@ -3577,7 +3577,7 @@
         <v>6</v>
       </c>
       <c r="N43">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O43">
         <v>6</v>
@@ -3615,7 +3615,7 @@
         <v>103</v>
       </c>
       <c r="D44">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E44">
         <v>1</v>
@@ -3636,7 +3636,7 @@
         <v>5</v>
       </c>
       <c r="K44">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L44">
         <v>5</v>
@@ -3689,13 +3689,13 @@
         <v>2</v>
       </c>
       <c r="F45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G45">
         <v>3</v>
       </c>
       <c r="H45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I45">
         <v>4</v>
@@ -3757,7 +3757,7 @@
         <v>4</v>
       </c>
       <c r="F46">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G46">
         <v>3</v>
@@ -3772,13 +3772,13 @@
         <v>5</v>
       </c>
       <c r="K46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L46">
         <v>4</v>
       </c>
       <c r="M46">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N46">
         <v>5</v>
@@ -3840,7 +3840,7 @@
         <v>6</v>
       </c>
       <c r="K47">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L47">
         <v>5</v>
@@ -3955,7 +3955,7 @@
         <v>103</v>
       </c>
       <c r="D49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E49">
         <v>1</v>
@@ -4035,7 +4035,7 @@
         <v>3</v>
       </c>
       <c r="H50">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I50">
         <v>3</v>
@@ -4050,7 +4050,7 @@
         <v>3</v>
       </c>
       <c r="M50">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N50">
         <v>4</v>
@@ -4100,7 +4100,7 @@
         <v>3</v>
       </c>
       <c r="G51">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H51">
         <v>2</v>
@@ -4112,13 +4112,13 @@
         <v>6</v>
       </c>
       <c r="K51">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L51">
         <v>6</v>
       </c>
       <c r="M51">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N51">
         <v>6</v>
@@ -4171,7 +4171,7 @@
         <v>2</v>
       </c>
       <c r="H52">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I52">
         <v>4</v>
@@ -4230,7 +4230,7 @@
         <v>2</v>
       </c>
       <c r="E53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F53">
         <v>2</v>
@@ -4245,7 +4245,7 @@
         <v>5</v>
       </c>
       <c r="J53">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K53">
         <v>5</v>
@@ -4254,7 +4254,7 @@
         <v>5</v>
       </c>
       <c r="M53">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N53">
         <v>5</v>
@@ -4298,7 +4298,7 @@
         <v>3</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F54">
         <v>3</v>
@@ -4307,22 +4307,22 @@
         <v>2</v>
       </c>
       <c r="H54">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I54">
         <v>3</v>
       </c>
       <c r="J54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K54">
         <v>3</v>
       </c>
       <c r="L54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M54">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N54">
         <v>3</v>
@@ -4381,7 +4381,7 @@
         <v>6</v>
       </c>
       <c r="J55">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K55">
         <v>5</v>
@@ -4443,7 +4443,7 @@
         <v>4</v>
       </c>
       <c r="H56">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I56">
         <v>4</v>
@@ -4514,10 +4514,10 @@
         <v>2</v>
       </c>
       <c r="I57">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J57">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K57">
         <v>6</v>
@@ -4529,7 +4529,7 @@
         <v>6</v>
       </c>
       <c r="N57">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O57">
         <v>6</v>
@@ -4579,7 +4579,7 @@
         <v>3</v>
       </c>
       <c r="H58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I58">
         <v>4</v>
@@ -4594,7 +4594,7 @@
         <v>5</v>
       </c>
       <c r="M58">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N58">
         <v>5</v>
@@ -4647,25 +4647,25 @@
         <v>2</v>
       </c>
       <c r="H59">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I59">
         <v>5</v>
       </c>
       <c r="J59">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K59">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L59">
         <v>4</v>
       </c>
       <c r="M59">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N59">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O59">
         <v>6</v>
@@ -4721,7 +4721,7 @@
         <v>5</v>
       </c>
       <c r="J60">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K60">
         <v>4</v>
@@ -4771,7 +4771,7 @@
         <v>103</v>
       </c>
       <c r="D61">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E61">
         <v>3</v>
@@ -4792,7 +4792,7 @@
         <v>4</v>
       </c>
       <c r="K61">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L61">
         <v>4</v>
@@ -4919,7 +4919,7 @@
         <v>4</v>
       </c>
       <c r="H63">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I63">
         <v>4</v>
@@ -4981,10 +4981,10 @@
         <v>2</v>
       </c>
       <c r="F64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H64">
         <v>3</v>
@@ -4993,19 +4993,19 @@
         <v>4</v>
       </c>
       <c r="J64">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K64">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L64">
         <v>5</v>
       </c>
       <c r="M64">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N64">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O64">
         <v>6</v>
@@ -5055,13 +5055,13 @@
         <v>2</v>
       </c>
       <c r="I65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J65">
         <v>6</v>
       </c>
       <c r="K65">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L65">
         <v>5</v>
@@ -5126,7 +5126,7 @@
         <v>4</v>
       </c>
       <c r="J66">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K66">
         <v>4</v>
@@ -5179,7 +5179,7 @@
         <v>2</v>
       </c>
       <c r="E67">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F67">
         <v>3</v>
@@ -5197,16 +5197,16 @@
         <v>6</v>
       </c>
       <c r="K67">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L67">
         <v>6</v>
       </c>
       <c r="M67">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N67">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O67">
         <v>6</v>
@@ -5268,7 +5268,7 @@
         <v>4</v>
       </c>
       <c r="L68">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M68">
         <v>4</v>
@@ -5315,13 +5315,13 @@
         <v>4</v>
       </c>
       <c r="E69">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F69">
         <v>5</v>
       </c>
       <c r="G69">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H69">
         <v>4</v>
@@ -5330,19 +5330,19 @@
         <v>3</v>
       </c>
       <c r="J69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K69">
         <v>4</v>
       </c>
       <c r="L69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M69">
         <v>3</v>
       </c>
       <c r="N69">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O69">
         <v>6</v>
@@ -5383,7 +5383,7 @@
         <v>2</v>
       </c>
       <c r="E70">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F70">
         <v>2</v>
@@ -5466,16 +5466,16 @@
         <v>6</v>
       </c>
       <c r="J71">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K71">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L71">
         <v>6</v>
       </c>
       <c r="M71">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N71">
         <v>6</v>
@@ -5516,10 +5516,10 @@
         <v>101</v>
       </c>
       <c r="D72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E72">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F72">
         <v>3</v>
@@ -5531,19 +5531,19 @@
         <v>4</v>
       </c>
       <c r="I72">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J72">
         <v>4</v>
       </c>
       <c r="K72">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L72">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M72">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N72">
         <v>4</v>
@@ -5587,7 +5587,7 @@
         <v>2</v>
       </c>
       <c r="E73">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F73">
         <v>2</v>
@@ -5605,7 +5605,7 @@
         <v>5</v>
       </c>
       <c r="K73">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L73">
         <v>5</v>
@@ -5655,13 +5655,13 @@
         <v>3</v>
       </c>
       <c r="E74">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F74">
         <v>4</v>
       </c>
       <c r="G74">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H74">
         <v>3</v>
@@ -5670,7 +5670,7 @@
         <v>4</v>
       </c>
       <c r="J74">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K74">
         <v>4</v>
@@ -5682,7 +5682,7 @@
         <v>4</v>
       </c>
       <c r="N74">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O74">
         <v>6</v>
@@ -5723,7 +5723,7 @@
         <v>2</v>
       </c>
       <c r="E75">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F75">
         <v>2</v>
@@ -5809,7 +5809,7 @@
         <v>4</v>
       </c>
       <c r="K76">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L76">
         <v>4</v>
@@ -5871,22 +5871,22 @@
         <v>4</v>
       </c>
       <c r="I77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K77">
         <v>4</v>
       </c>
       <c r="L77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M77">
         <v>3</v>
       </c>
       <c r="N77">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O77">
         <v>6</v>
@@ -5924,7 +5924,7 @@
         <v>103</v>
       </c>
       <c r="D78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E78">
         <v>2</v>
@@ -5954,7 +5954,7 @@
         <v>6</v>
       </c>
       <c r="N78">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O78">
         <v>6</v>
@@ -5998,31 +5998,31 @@
         <v>3</v>
       </c>
       <c r="F79">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G79">
         <v>2</v>
       </c>
       <c r="H79">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I79">
         <v>4</v>
       </c>
       <c r="J79">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K79">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L79">
         <v>4</v>
       </c>
       <c r="M79">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N79">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="O79">
         <v>6</v>
@@ -6084,7 +6084,7 @@
         <v>4</v>
       </c>
       <c r="L80">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M80">
         <v>4</v>

</xml_diff>